<commit_message>
Add SE tax reserve, sinking funds, income trajectory, and savings goals
New sections on The System tab: self-employment tax reserve (28% of $480
side work = $134/mo, formula-driven); sinking funds (truck maintenance
$75, registration $17, insurance placeholder); income trajectory ($11.81
effective → $22 target → ~$414/mo gain); savings goals in sequence
(Emergency Fund $7k then Septic Fund $7,285, both with current/remaining/%
complete driven by a single blue input cell); revised bottom line showing
true monthly available after all deductions and Shane contingency floor.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019a94zwuEHMtxW31Vn2e8yf
</commit_message>
<xml_diff>
--- a/utilities/Budget_System.xlsx
+++ b/utilities/Budget_System.xlsx
@@ -19,11 +19,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00;[Red]-&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00;[Red]-&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -59,6 +60,18 @@
       <b val="1"/>
       <color rgb="001E293B"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="002563EB"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="002563EB"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -116,7 +129,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="16">
+  <fills count="19">
     <fill>
       <patternFill/>
     </fill>
@@ -170,6 +183,21 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="007C3AED"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDE9FE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DBEAFE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="000EA5E9"/>
       </patternFill>
     </fill>
@@ -206,7 +234,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="76">
+  <cellXfs count="90">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -278,73 +306,115 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="11" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="12" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="10" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="11" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="12" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="10" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -353,76 +423,76 @@
     <xf numFmtId="164" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="16" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="11" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="16" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="11" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="17" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="15" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="17" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -973,7 +1043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D41"/>
+  <dimension ref="A1:D79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1402,14 +1472,421 @@
       </c>
       <c r="D41" s="26" t="n"/>
     </row>
+    <row r="42" ht="8" customHeight="1"/>
+    <row r="43" ht="22" customHeight="1">
+      <c r="A43" s="27" t="inlineStr">
+        <is>
+          <t>SELF-EMPLOYMENT TAX RESERVE  (1099 side work)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="20" customHeight="1">
+      <c r="B44" s="12" t="inlineStr">
+        <is>
+          <t>Side work gross  (from income above)</t>
+        </is>
+      </c>
+      <c r="C44" s="13">
+        <f>C6</f>
+        <v/>
+      </c>
+      <c r="D44" s="16" t="inlineStr">
+        <is>
+          <t>1099 — no taxes withheld; this must come out before you touch the money</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="20" customHeight="1">
+      <c r="B45" s="28" t="inlineStr">
+        <is>
+          <t>Monthly reserve  (28% — SE tax 15.3% + income tax est.)</t>
+        </is>
+      </c>
+      <c r="C45" s="29">
+        <f>C44*0.28</f>
+        <v/>
+      </c>
+      <c r="D45" s="30" t="inlineStr">
+        <is>
+          <t>Transfer on every payday before spending any side income</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="20" customHeight="1">
+      <c r="B46" s="12" t="inlineStr">
+        <is>
+          <t>True spendable from side work</t>
+        </is>
+      </c>
+      <c r="C46" s="13">
+        <f>C44-C45</f>
+        <v/>
+      </c>
+      <c r="D46" s="16" t="inlineStr">
+        <is>
+          <t>What's actually yours after the tax reserve is parked</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="8" customHeight="1"/>
+    <row r="48" ht="22" customHeight="1">
+      <c r="A48" s="15" t="inlineStr">
+        <is>
+          <t>SINKING FUNDS  — annual / irregular costs ÷ 12</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="20" customHeight="1">
+      <c r="B49" s="12" t="inlineStr">
+        <is>
+          <t>Truck maintenance  (1999 Silverado, self-maintained)</t>
+        </is>
+      </c>
+      <c r="C49" s="13" t="n">
+        <v>75</v>
+      </c>
+      <c r="D49" s="16" t="inlineStr">
+        <is>
+          <t>~$900/yr est. · adjust to your history</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="20" customHeight="1">
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>Vehicle registration  (AL, annual)</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="D50" s="6" t="inlineStr">
+        <is>
+          <t>~$200/yr ÷ 12</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="20" customHeight="1">
+      <c r="B51" s="12" t="inlineStr">
+        <is>
+          <t>Annual insurance premiums  (if any lump-sum)</t>
+        </is>
+      </c>
+      <c r="C51" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D51" s="16" t="inlineStr">
+        <is>
+          <t>$0 if already paying monthly — update if any biller charges annually</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="20" customHeight="1">
+      <c r="B52" s="7" t="inlineStr">
+        <is>
+          <t>SINKING TOTAL  — set aside monthly</t>
+        </is>
+      </c>
+      <c r="C52" s="8">
+        <f>SUM(C49:C51)</f>
+        <v/>
+      </c>
+      <c r="D52" s="31" t="inlineStr">
+        <is>
+          <t>Park in a labeled savings vault; pull from it when the bill hits</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="8" customHeight="1"/>
+    <row r="54" ht="22" customHeight="1">
+      <c r="A54" s="11" t="inlineStr">
+        <is>
+          <t>INCOME TRAJECTORY  — current effective wage → target</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="20" customHeight="1">
+      <c r="B55" s="12" t="inlineStr">
+        <is>
+          <t>Current effective wage  (50hr wk + 7hr commute)</t>
+        </is>
+      </c>
+      <c r="C55" s="32" t="n">
+        <v>11.81</v>
+      </c>
+      <c r="D55" s="16" t="inlineStr">
+        <is>
+          <t>$2,560 take-home ÷ ~217 hrs/mo (50hr work + 7hr commute = ~7hr/day)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="20" customHeight="1">
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>Current monthly take-home  (Coke only)</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="n">
+        <v>2560</v>
+      </c>
+      <c r="D56" s="6" t="inlineStr">
+        <is>
+          <t>Baseline — side work net is on top of this</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="20" customHeight="1">
+      <c r="B57" s="12" t="inlineStr">
+        <is>
+          <t>Target wage after retraining  ($20–25/hr, $22 midpoint)</t>
+        </is>
+      </c>
+      <c r="C57" s="32" t="n">
+        <v>22</v>
+      </c>
+      <c r="D57" s="16" t="inlineStr">
+        <is>
+          <t>Midpoint of stated $20–25/hr range</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="20" customHeight="1">
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>Est. take-home at $22/hr  (40hr/wk, ~72% net)</t>
+        </is>
+      </c>
+      <c r="C58" s="5">
+        <f>22*40*52/12*0.72</f>
+        <v/>
+      </c>
+      <c r="D58" s="6" t="inlineStr">
+        <is>
+          <t>Rough estimate — actual varies by deductions</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="20" customHeight="1">
+      <c r="B59" s="24" t="inlineStr">
+        <is>
+          <t>Monthly income gain at target</t>
+        </is>
+      </c>
+      <c r="C59" s="25">
+        <f>C58-C56</f>
+        <v/>
+      </c>
+      <c r="D59" s="23" t="inlineStr">
+        <is>
+          <t>Extra per month once you land the better role</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="8" customHeight="1"/>
+    <row r="61" ht="22" customHeight="1">
+      <c r="A61" s="17" t="inlineStr">
+        <is>
+          <t>SAVINGS GOALS  (sequential — ① Emergency Fund first)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="22" customHeight="1">
+      <c r="A62" s="33" t="inlineStr">
+        <is>
+          <t>Current savings balance  ← UPDATE THIS INPUT</t>
+        </is>
+      </c>
+      <c r="C62" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="D62" s="35" t="inlineStr">
+        <is>
+          <t>Blue = input cell  ·  enter your actual savings balance here</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="6" customHeight="1"/>
+    <row r="64" ht="20" customHeight="1">
+      <c r="B64" s="36" t="inlineStr">
+        <is>
+          <t>① EMERGENCY FUND — target</t>
+        </is>
+      </c>
+      <c r="C64" s="37" t="n">
+        <v>7000</v>
+      </c>
+      <c r="D64" s="14" t="n"/>
+    </row>
+    <row r="65" ht="20" customHeight="1">
+      <c r="B65" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Current  (from balance above)</t>
+        </is>
+      </c>
+      <c r="C65" s="13">
+        <f>MIN(C62,7000)</f>
+        <v/>
+      </c>
+      <c r="D65" s="14" t="n"/>
+    </row>
+    <row r="66" ht="20" customHeight="1">
+      <c r="B66" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Remaining</t>
+        </is>
+      </c>
+      <c r="C66" s="13">
+        <f>MAX(0,C64-C65)</f>
+        <v/>
+      </c>
+      <c r="D66" s="14" t="n"/>
+    </row>
+    <row r="67" ht="20" customHeight="1">
+      <c r="B67" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   % Complete</t>
+        </is>
+      </c>
+      <c r="C67" s="38">
+        <f>IFERROR(C65/C64,0)</f>
+        <v/>
+      </c>
+      <c r="D67" s="26" t="n"/>
+    </row>
+    <row r="68" ht="6" customHeight="1"/>
+    <row r="69" ht="20" customHeight="1">
+      <c r="B69" s="39" t="inlineStr">
+        <is>
+          <t>② SEPTIC FUND — target  (starts after EF hits $7,000)</t>
+        </is>
+      </c>
+      <c r="C69" s="40" t="n">
+        <v>7285</v>
+      </c>
+      <c r="D69" s="10" t="n"/>
+    </row>
+    <row r="70" ht="20" customHeight="1">
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Current  (balance above − $7,000 EF)</t>
+        </is>
+      </c>
+      <c r="C70" s="5">
+        <f>MAX(0,C62-7000)</f>
+        <v/>
+      </c>
+      <c r="D70" s="10" t="n"/>
+    </row>
+    <row r="71" ht="20" customHeight="1">
+      <c r="B71" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Remaining</t>
+        </is>
+      </c>
+      <c r="C71" s="13">
+        <f>MAX(0,C69-C70)</f>
+        <v/>
+      </c>
+      <c r="D71" s="14" t="n"/>
+    </row>
+    <row r="72" ht="20" customHeight="1">
+      <c r="B72" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   % Complete</t>
+        </is>
+      </c>
+      <c r="C72" s="38">
+        <f>IFERROR(C70/C69,0)</f>
+        <v/>
+      </c>
+      <c r="D72" s="26" t="n"/>
+    </row>
+    <row r="73" ht="8" customHeight="1"/>
+    <row r="74" ht="22" customHeight="1">
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t>REVISED MONTHLY PICTURE  (after tax reserve + sinking funds)</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="20" customHeight="1">
+      <c r="B75" s="12" t="inlineStr">
+        <is>
+          <t>Gross leftover  (after fixed + flex)</t>
+        </is>
+      </c>
+      <c r="C75" s="13">
+        <f>C31</f>
+        <v/>
+      </c>
+      <c r="D75" s="14" t="n"/>
+    </row>
+    <row r="76" ht="20" customHeight="1">
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Less: SE tax reserve</t>
+        </is>
+      </c>
+      <c r="C76" s="5">
+        <f>-C45</f>
+        <v/>
+      </c>
+      <c r="D76" s="10" t="n"/>
+    </row>
+    <row r="77" ht="20" customHeight="1">
+      <c r="B77" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Less: sinking funds</t>
+        </is>
+      </c>
+      <c r="C77" s="13">
+        <f>-C52</f>
+        <v/>
+      </c>
+      <c r="D77" s="14" t="n"/>
+    </row>
+    <row r="78" ht="20" customHeight="1">
+      <c r="B78" s="7" t="inlineStr">
+        <is>
+          <t>TRUE MONTHLY AVAILABLE</t>
+        </is>
+      </c>
+      <c r="C78" s="8">
+        <f>C31-C45-C52</f>
+        <v/>
+      </c>
+      <c r="D78" s="9" t="n"/>
+    </row>
+    <row r="79" ht="20" customHeight="1">
+      <c r="B79" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  If Shane's $628 stops → true available</t>
+        </is>
+      </c>
+      <c r="C79" s="19">
+        <f>C78-628</f>
+        <v/>
+      </c>
+      <c r="D79" s="20" t="inlineStr">
+        <is>
+          <t>Hard number — build the system around this floor</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="14">
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A62:B62"/>
+    <mergeCell ref="A61:D61"/>
+    <mergeCell ref="A74:D74"/>
     <mergeCell ref="A11:D11"/>
     <mergeCell ref="A34:D34"/>
     <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A48:D48"/>
     <mergeCell ref="A30:D30"/>
     <mergeCell ref="A38:D38"/>
+    <mergeCell ref="A54:D54"/>
+    <mergeCell ref="A43:D43"/>
     <mergeCell ref="A19:D19"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
@@ -1440,7 +1917,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="27" t="inlineStr">
+      <c r="A1" s="41" t="inlineStr">
         <is>
           <t>MONTHLY CHECK-IN &amp; SWEEP LOG</t>
         </is>
@@ -1454,1183 +1931,1183 @@
       </c>
     </row>
     <row r="4" ht="28" customHeight="1">
-      <c r="A4" s="28" t="inlineStr">
+      <c r="A4" s="42" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B4" s="29" t="inlineStr">
+      <c r="B4" s="43" t="inlineStr">
         <is>
           <t>Water</t>
         </is>
       </c>
-      <c r="C4" s="30" t="inlineStr">
+      <c r="C4" s="44" t="inlineStr">
         <is>
           <t>Power</t>
         </is>
       </c>
-      <c r="D4" s="31" t="inlineStr">
+      <c r="D4" s="45" t="inlineStr">
         <is>
           <t>Internet</t>
         </is>
       </c>
-      <c r="E4" s="32" t="inlineStr">
+      <c r="E4" s="46" t="inlineStr">
         <is>
           <t>Trash</t>
         </is>
       </c>
-      <c r="F4" s="28" t="inlineStr">
+      <c r="F4" s="42" t="inlineStr">
         <is>
           <t>Total Actual</t>
         </is>
       </c>
-      <c r="G4" s="33" t="inlineStr">
+      <c r="G4" s="47" t="inlineStr">
         <is>
           <t>Funded</t>
         </is>
       </c>
-      <c r="H4" s="34" t="inlineStr">
+      <c r="H4" s="48" t="inlineStr">
         <is>
           <t>Net  (+/−)</t>
         </is>
       </c>
-      <c r="I4" s="35" t="inlineStr">
+      <c r="I4" s="49" t="inlineStr">
         <is>
           <t>Buffer Bal</t>
         </is>
       </c>
-      <c r="J4" s="36" t="inlineStr">
+      <c r="J4" s="50" t="inlineStr">
         <is>
           <t>→ Savings</t>
         </is>
       </c>
-      <c r="K4" s="28" t="inlineStr">
+      <c r="K4" s="42" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="37" t="inlineStr">
+      <c r="A5" s="51" t="inlineStr">
         <is>
           <t>Jun '25</t>
         </is>
       </c>
-      <c r="B5" s="38" t="n">
+      <c r="B5" s="52" t="n">
         <v>22.5</v>
       </c>
-      <c r="C5" s="38" t="n">
+      <c r="C5" s="52" t="n">
         <v>368.62</v>
       </c>
-      <c r="D5" s="38" t="n">
+      <c r="D5" s="52" t="n">
         <v>42.97</v>
       </c>
-      <c r="E5" s="38" t="n">
+      <c r="E5" s="52" t="n">
         <v>21.37</v>
       </c>
-      <c r="F5" s="39">
+      <c r="F5" s="53">
         <f>IFERROR(SUM(B5:E5),"")</f>
         <v/>
       </c>
-      <c r="G5" s="40" t="n">
+      <c r="G5" s="54" t="n">
         <v>630</v>
       </c>
-      <c r="H5" s="41">
+      <c r="H5" s="55">
         <f>IFERROR(G5-F5,"")</f>
         <v/>
       </c>
-      <c r="I5" s="38">
+      <c r="I5" s="52">
         <f>IFERROR(MAX(0,MIN(167.63,167.63+H5)),"")</f>
         <v/>
       </c>
-      <c r="J5" s="42">
+      <c r="J5" s="56">
         <f>IFERROR(MAX(0,H5-MAX(0,167.63-167.63)),"")</f>
         <v/>
       </c>
-      <c r="K5" s="43" t="n"/>
+      <c r="K5" s="57" t="n"/>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="44" t="inlineStr">
+      <c r="A6" s="58" t="inlineStr">
         <is>
           <t>Jul '25</t>
         </is>
       </c>
-      <c r="B6" s="45" t="n">
+      <c r="B6" s="59" t="n">
         <v>28.32</v>
       </c>
-      <c r="C6" s="45" t="n">
+      <c r="C6" s="59" t="n">
         <v>440.17</v>
       </c>
-      <c r="D6" s="45" t="n">
+      <c r="D6" s="59" t="n">
         <v>42.98</v>
       </c>
-      <c r="E6" s="45" t="n">
+      <c r="E6" s="59" t="n">
         <v>24.77</v>
       </c>
-      <c r="F6" s="46">
+      <c r="F6" s="60">
         <f>IFERROR(SUM(B6:E6),"")</f>
         <v/>
       </c>
-      <c r="G6" s="47" t="n">
+      <c r="G6" s="61" t="n">
         <v>630</v>
       </c>
-      <c r="H6" s="48">
+      <c r="H6" s="62">
         <f>IFERROR(G6-F6,"")</f>
         <v/>
       </c>
-      <c r="I6" s="45">
+      <c r="I6" s="59">
         <f>IFERROR(MAX(0,MIN(167.63,I5+H6)),"")</f>
         <v/>
       </c>
-      <c r="J6" s="49">
+      <c r="J6" s="63">
         <f>IFERROR(MAX(0,H6-MAX(0,167.63-167.63)),"")</f>
         <v/>
       </c>
       <c r="K6" s="2" t="n"/>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="37" t="inlineStr">
+      <c r="A7" s="51" t="inlineStr">
         <is>
           <t>Aug '25</t>
         </is>
       </c>
-      <c r="B7" s="38" t="n">
+      <c r="B7" s="52" t="n">
         <v>24.35</v>
       </c>
-      <c r="C7" s="38" t="n">
+      <c r="C7" s="52" t="n">
         <v>429.27</v>
       </c>
-      <c r="D7" s="38" t="n">
+      <c r="D7" s="52" t="n">
         <v>42.98</v>
       </c>
-      <c r="E7" s="38" t="n"/>
-      <c r="F7" s="39">
+      <c r="E7" s="52" t="n"/>
+      <c r="F7" s="53">
         <f>IFERROR(SUM(B7:E7),"")</f>
         <v/>
       </c>
-      <c r="G7" s="40" t="n">
+      <c r="G7" s="54" t="n">
         <v>630</v>
       </c>
-      <c r="H7" s="41">
+      <c r="H7" s="55">
         <f>IFERROR(G7-F7,"")</f>
         <v/>
       </c>
-      <c r="I7" s="38">
+      <c r="I7" s="52">
         <f>IFERROR(MAX(0,MIN(167.63,I6+H7)),"")</f>
         <v/>
       </c>
-      <c r="J7" s="42">
+      <c r="J7" s="56">
         <f>IFERROR(MAX(0,H7-MAX(0,167.63-167.63)),"")</f>
         <v/>
       </c>
-      <c r="K7" s="43" t="n"/>
+      <c r="K7" s="57" t="n"/>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="44" t="inlineStr">
+      <c r="A8" s="58" t="inlineStr">
         <is>
           <t>Sep '25</t>
         </is>
       </c>
-      <c r="B8" s="45" t="n">
+      <c r="B8" s="59" t="n">
         <v>33.54</v>
       </c>
-      <c r="C8" s="45" t="n">
+      <c r="C8" s="59" t="n">
         <v>381.57</v>
       </c>
-      <c r="D8" s="45" t="n">
+      <c r="D8" s="59" t="n">
         <v>63.03</v>
       </c>
-      <c r="E8" s="45" t="n">
+      <c r="E8" s="59" t="n">
         <v>21.37</v>
       </c>
-      <c r="F8" s="46">
+      <c r="F8" s="60">
         <f>IFERROR(SUM(B8:E8),"")</f>
         <v/>
       </c>
-      <c r="G8" s="47" t="n">
+      <c r="G8" s="61" t="n">
         <v>630</v>
       </c>
-      <c r="H8" s="48">
+      <c r="H8" s="62">
         <f>IFERROR(G8-F8,"")</f>
         <v/>
       </c>
-      <c r="I8" s="45">
+      <c r="I8" s="59">
         <f>IFERROR(MAX(0,MIN(167.63,I7+H8)),"")</f>
         <v/>
       </c>
-      <c r="J8" s="49">
+      <c r="J8" s="63">
         <f>IFERROR(MAX(0,H8-MAX(0,167.63-167.63)),"")</f>
         <v/>
       </c>
       <c r="K8" s="2" t="n"/>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="37" t="inlineStr">
+      <c r="A9" s="51" t="inlineStr">
         <is>
           <t>Oct '25</t>
         </is>
       </c>
-      <c r="B9" s="38" t="n">
+      <c r="B9" s="52" t="n">
         <v>35.97</v>
       </c>
-      <c r="C9" s="38" t="n">
+      <c r="C9" s="52" t="n">
         <v>248.35</v>
       </c>
-      <c r="D9" s="38" t="n">
+      <c r="D9" s="52" t="n">
         <v>63.03</v>
       </c>
-      <c r="E9" s="38" t="n">
+      <c r="E9" s="52" t="n">
         <v>21.37</v>
       </c>
-      <c r="F9" s="39">
+      <c r="F9" s="53">
         <f>IFERROR(SUM(B9:E9),"")</f>
         <v/>
       </c>
-      <c r="G9" s="40" t="n">
+      <c r="G9" s="54" t="n">
         <v>630</v>
       </c>
-      <c r="H9" s="41">
+      <c r="H9" s="55">
         <f>IFERROR(G9-F9,"")</f>
         <v/>
       </c>
-      <c r="I9" s="38">
+      <c r="I9" s="52">
         <f>IFERROR(MAX(0,MIN(167.63,I8+H9)),"")</f>
         <v/>
       </c>
-      <c r="J9" s="42">
+      <c r="J9" s="56">
         <f>IFERROR(MAX(0,H9-MAX(0,167.63-167.63)),"")</f>
         <v/>
       </c>
-      <c r="K9" s="43" t="n"/>
+      <c r="K9" s="57" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="44" t="inlineStr">
+      <c r="A10" s="58" t="inlineStr">
         <is>
           <t>Nov '25</t>
         </is>
       </c>
-      <c r="B10" s="45" t="n">
+      <c r="B10" s="59" t="n">
         <v>35.97</v>
       </c>
-      <c r="C10" s="45" t="n">
+      <c r="C10" s="59" t="n">
         <v>264.5</v>
       </c>
-      <c r="D10" s="45" t="n">
+      <c r="D10" s="59" t="n">
         <v>63.03</v>
       </c>
-      <c r="E10" s="45" t="n">
+      <c r="E10" s="59" t="n">
         <v>21.37</v>
       </c>
-      <c r="F10" s="46">
+      <c r="F10" s="60">
         <f>IFERROR(SUM(B10:E10),"")</f>
         <v/>
       </c>
-      <c r="G10" s="47" t="n">
+      <c r="G10" s="61" t="n">
         <v>630</v>
       </c>
-      <c r="H10" s="48">
+      <c r="H10" s="62">
         <f>IFERROR(G10-F10,"")</f>
         <v/>
       </c>
-      <c r="I10" s="45">
+      <c r="I10" s="59">
         <f>IFERROR(MAX(0,MIN(167.63,I9+H10)),"")</f>
         <v/>
       </c>
-      <c r="J10" s="49">
+      <c r="J10" s="63">
         <f>IFERROR(MAX(0,H10-MAX(0,167.63-167.63)),"")</f>
         <v/>
       </c>
       <c r="K10" s="2" t="n"/>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="37" t="inlineStr">
+      <c r="A11" s="51" t="inlineStr">
         <is>
           <t>Dec '25</t>
         </is>
       </c>
-      <c r="B11" s="38" t="n">
+      <c r="B11" s="52" t="n">
         <v>44.13</v>
       </c>
-      <c r="C11" s="38" t="n">
+      <c r="C11" s="52" t="n">
         <v>415.04</v>
       </c>
-      <c r="D11" s="38" t="n">
+      <c r="D11" s="52" t="n">
         <v>63.03</v>
       </c>
-      <c r="E11" s="38" t="n">
+      <c r="E11" s="52" t="n">
         <v>21.37</v>
       </c>
-      <c r="F11" s="39">
+      <c r="F11" s="53">
         <f>IFERROR(SUM(B11:E11),"")</f>
         <v/>
       </c>
-      <c r="G11" s="40" t="n">
+      <c r="G11" s="54" t="n">
         <v>630</v>
       </c>
-      <c r="H11" s="41">
+      <c r="H11" s="55">
         <f>IFERROR(G11-F11,"")</f>
         <v/>
       </c>
-      <c r="I11" s="38">
+      <c r="I11" s="52">
         <f>IFERROR(MAX(0,MIN(167.63,I10+H11)),"")</f>
         <v/>
       </c>
-      <c r="J11" s="42">
+      <c r="J11" s="56">
         <f>IFERROR(MAX(0,H11-MAX(0,167.63-167.63)),"")</f>
         <v/>
       </c>
-      <c r="K11" s="43" t="n"/>
+      <c r="K11" s="57" t="n"/>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="44" t="inlineStr">
+      <c r="A12" s="58" t="inlineStr">
         <is>
           <t>Jan '26</t>
         </is>
       </c>
-      <c r="B12" s="45" t="n">
+      <c r="B12" s="59" t="n">
         <v>40.52</v>
       </c>
-      <c r="C12" s="45" t="n">
+      <c r="C12" s="59" t="n">
         <v>541.9</v>
       </c>
-      <c r="D12" s="45" t="n">
+      <c r="D12" s="59" t="n">
         <v>24.95</v>
       </c>
-      <c r="E12" s="45" t="n">
+      <c r="E12" s="59" t="n">
         <v>22.01</v>
       </c>
-      <c r="F12" s="46">
+      <c r="F12" s="60">
         <f>IFERROR(SUM(B12:E12),"")</f>
         <v/>
       </c>
-      <c r="G12" s="47" t="n">
+      <c r="G12" s="61" t="n">
         <v>630</v>
       </c>
-      <c r="H12" s="48">
+      <c r="H12" s="62">
         <f>IFERROR(G12-F12,"")</f>
         <v/>
       </c>
-      <c r="I12" s="45">
+      <c r="I12" s="59">
         <f>IFERROR(MAX(0,MIN(167.63,I11+H12)),"")</f>
         <v/>
       </c>
-      <c r="J12" s="49">
+      <c r="J12" s="63">
         <f>IFERROR(MAX(0,H12-MAX(0,167.63-167.63)),"")</f>
         <v/>
       </c>
       <c r="K12" s="2" t="n"/>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="37" t="inlineStr">
+      <c r="A13" s="51" t="inlineStr">
         <is>
           <t>Feb '26</t>
         </is>
       </c>
-      <c r="B13" s="38" t="n">
+      <c r="B13" s="52" t="n">
         <v>31.02</v>
       </c>
-      <c r="C13" s="38" t="n">
+      <c r="C13" s="52" t="n">
         <v>388.23</v>
       </c>
-      <c r="D13" s="38" t="n">
+      <c r="D13" s="52" t="n">
         <v>24.95</v>
       </c>
-      <c r="E13" s="38" t="n">
+      <c r="E13" s="52" t="n">
         <v>22.01</v>
       </c>
-      <c r="F13" s="39">
+      <c r="F13" s="53">
         <f>IFERROR(SUM(B13:E13),"")</f>
         <v/>
       </c>
-      <c r="G13" s="40" t="n">
+      <c r="G13" s="54" t="n">
         <v>630</v>
       </c>
-      <c r="H13" s="41">
+      <c r="H13" s="55">
         <f>IFERROR(G13-F13,"")</f>
         <v/>
       </c>
-      <c r="I13" s="38">
+      <c r="I13" s="52">
         <f>IFERROR(MAX(0,MIN(167.63,I12+H13)),"")</f>
         <v/>
       </c>
-      <c r="J13" s="42">
+      <c r="J13" s="56">
         <f>IFERROR(MAX(0,H13-MAX(0,167.63-167.63)),"")</f>
         <v/>
       </c>
-      <c r="K13" s="43" t="n"/>
+      <c r="K13" s="57" t="n"/>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="44" t="inlineStr">
+      <c r="A14" s="58" t="inlineStr">
         <is>
           <t>Mar '26</t>
         </is>
       </c>
-      <c r="B14" s="45" t="n">
+      <c r="B14" s="59" t="n">
         <v>39.61</v>
       </c>
-      <c r="C14" s="45" t="n">
+      <c r="C14" s="59" t="n">
         <v>226.71</v>
       </c>
-      <c r="D14" s="45" t="n">
+      <c r="D14" s="59" t="n">
         <v>24.95</v>
       </c>
-      <c r="E14" s="45" t="n">
+      <c r="E14" s="59" t="n">
         <v>22.01</v>
       </c>
-      <c r="F14" s="46">
+      <c r="F14" s="60">
         <f>IFERROR(SUM(B14:E14),"")</f>
         <v/>
       </c>
-      <c r="G14" s="47" t="n">
+      <c r="G14" s="61" t="n">
         <v>630</v>
       </c>
-      <c r="H14" s="48">
+      <c r="H14" s="62">
         <f>IFERROR(G14-F14,"")</f>
         <v/>
       </c>
-      <c r="I14" s="45">
+      <c r="I14" s="59">
         <f>IFERROR(MAX(0,MIN(167.63,I13+H14)),"")</f>
         <v/>
       </c>
-      <c r="J14" s="49">
+      <c r="J14" s="63">
         <f>IFERROR(MAX(0,H14-MAX(0,167.63-167.63)),"")</f>
         <v/>
       </c>
       <c r="K14" s="2" t="n"/>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="37" t="inlineStr">
+      <c r="A15" s="51" t="inlineStr">
         <is>
           <t>Apr '26</t>
         </is>
       </c>
-      <c r="B15" s="38" t="n">
+      <c r="B15" s="52" t="n">
         <v>86.5</v>
       </c>
-      <c r="C15" s="38" t="n">
+      <c r="C15" s="52" t="n">
         <v>206.01</v>
       </c>
-      <c r="D15" s="38" t="n">
+      <c r="D15" s="52" t="n">
         <v>24.95</v>
       </c>
-      <c r="E15" s="38" t="n">
+      <c r="E15" s="52" t="n">
         <v>22.01</v>
       </c>
-      <c r="F15" s="39">
+      <c r="F15" s="53">
         <f>IFERROR(SUM(B15:E15),"")</f>
         <v/>
       </c>
-      <c r="G15" s="40" t="n">
+      <c r="G15" s="54" t="n">
         <v>630</v>
       </c>
-      <c r="H15" s="41">
+      <c r="H15" s="55">
         <f>IFERROR(G15-F15,"")</f>
         <v/>
       </c>
-      <c r="I15" s="38">
+      <c r="I15" s="52">
         <f>IFERROR(MAX(0,MIN(167.63,I14+H15)),"")</f>
         <v/>
       </c>
-      <c r="J15" s="42">
+      <c r="J15" s="56">
         <f>IFERROR(MAX(0,H15-MAX(0,167.63-167.63)),"")</f>
         <v/>
       </c>
-      <c r="K15" s="43" t="n"/>
+      <c r="K15" s="57" t="n"/>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="44" t="inlineStr">
+      <c r="A16" s="58" t="inlineStr">
         <is>
           <t>May '26</t>
         </is>
       </c>
-      <c r="B16" s="45" t="n"/>
-      <c r="C16" s="45" t="n"/>
-      <c r="D16" s="45" t="n"/>
-      <c r="E16" s="45" t="n"/>
-      <c r="F16" s="46">
+      <c r="B16" s="59" t="n"/>
+      <c r="C16" s="59" t="n"/>
+      <c r="D16" s="59" t="n"/>
+      <c r="E16" s="59" t="n"/>
+      <c r="F16" s="60">
         <f>IFERROR(SUM(B16:E16),"")</f>
         <v/>
       </c>
-      <c r="G16" s="47" t="n">
+      <c r="G16" s="61" t="n">
         <v>630</v>
       </c>
-      <c r="H16" s="48">
+      <c r="H16" s="62">
         <f>IFERROR(G16-F16,"")</f>
         <v/>
       </c>
-      <c r="I16" s="45">
+      <c r="I16" s="59">
         <f>IFERROR(MAX(0,MIN(167.63,I15+H16)),"")</f>
         <v/>
       </c>
-      <c r="J16" s="49">
+      <c r="J16" s="63">
         <f>IFERROR(MAX(0,H16-MAX(0,167.63-167.63)),"")</f>
         <v/>
       </c>
       <c r="K16" s="2" t="n"/>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="37" t="inlineStr">
+      <c r="A17" s="51" t="inlineStr">
         <is>
           <t>Jun '26</t>
         </is>
       </c>
-      <c r="B17" s="38" t="n">
+      <c r="B17" s="52" t="n">
         <v>166.96</v>
       </c>
-      <c r="C17" s="38" t="n">
+      <c r="C17" s="52" t="n">
         <v>220.59</v>
       </c>
-      <c r="D17" s="38" t="n">
+      <c r="D17" s="52" t="n">
         <v>24.95</v>
       </c>
-      <c r="E17" s="38" t="n">
+      <c r="E17" s="52" t="n">
         <v>22.01</v>
       </c>
-      <c r="F17" s="39">
+      <c r="F17" s="53">
         <f>IFERROR(SUM(B17:E17),"")</f>
         <v/>
       </c>
-      <c r="G17" s="40" t="n">
+      <c r="G17" s="54" t="n">
         <v>630</v>
       </c>
-      <c r="H17" s="41">
+      <c r="H17" s="55">
         <f>IFERROR(G17-F17,"")</f>
         <v/>
       </c>
-      <c r="I17" s="38">
+      <c r="I17" s="52">
         <f>IFERROR(MAX(0,MIN(167.63,I16+H17)),"")</f>
         <v/>
       </c>
-      <c r="J17" s="42">
+      <c r="J17" s="56">
         <f>IFERROR(MAX(0,H17-MAX(0,167.63-167.63)),"")</f>
         <v/>
       </c>
-      <c r="K17" s="43" t="n"/>
+      <c r="K17" s="57" t="n"/>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="44" t="inlineStr">
+      <c r="A18" s="58" t="inlineStr">
         <is>
           <t>Jul '26</t>
         </is>
       </c>
-      <c r="B18" s="45" t="n"/>
-      <c r="C18" s="45" t="n"/>
-      <c r="D18" s="45" t="n"/>
-      <c r="E18" s="45" t="n"/>
-      <c r="F18" s="46">
+      <c r="B18" s="59" t="n"/>
+      <c r="C18" s="59" t="n"/>
+      <c r="D18" s="59" t="n"/>
+      <c r="E18" s="59" t="n"/>
+      <c r="F18" s="60">
         <f>IFERROR(SUM(B18:E18),"")</f>
         <v/>
       </c>
-      <c r="G18" s="47" t="n">
+      <c r="G18" s="61" t="n">
         <v>630</v>
       </c>
-      <c r="H18" s="48">
+      <c r="H18" s="62">
         <f>IFERROR(G18-F18,"")</f>
         <v/>
       </c>
-      <c r="I18" s="45">
+      <c r="I18" s="59">
         <f>IFERROR(MAX(0,MIN(167.63,I17+H18)),"")</f>
         <v/>
       </c>
-      <c r="J18" s="49">
+      <c r="J18" s="63">
         <f>IFERROR(MAX(0,H18-MAX(0,167.63-167.63)),"")</f>
         <v/>
       </c>
       <c r="K18" s="2" t="n"/>
     </row>
     <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="37" t="inlineStr">
+      <c r="A19" s="51" t="inlineStr">
         <is>
           <t>Aug '26</t>
         </is>
       </c>
-      <c r="B19" s="38" t="n"/>
-      <c r="C19" s="38" t="n"/>
-      <c r="D19" s="38" t="n"/>
-      <c r="E19" s="38" t="n"/>
-      <c r="F19" s="39">
+      <c r="B19" s="52" t="n"/>
+      <c r="C19" s="52" t="n"/>
+      <c r="D19" s="52" t="n"/>
+      <c r="E19" s="52" t="n"/>
+      <c r="F19" s="53">
         <f>IFERROR(SUM(B19:E19),"")</f>
         <v/>
       </c>
-      <c r="G19" s="40" t="n">
+      <c r="G19" s="54" t="n">
         <v>630</v>
       </c>
-      <c r="H19" s="41">
+      <c r="H19" s="55">
         <f>IFERROR(G19-F19,"")</f>
         <v/>
       </c>
-      <c r="I19" s="38">
+      <c r="I19" s="52">
         <f>IFERROR(MAX(0,MIN(167.63,I18+H19)),"")</f>
         <v/>
       </c>
-      <c r="J19" s="42">
+      <c r="J19" s="56">
         <f>IFERROR(MAX(0,H19-MAX(0,167.63-167.63)),"")</f>
         <v/>
       </c>
-      <c r="K19" s="43" t="n"/>
+      <c r="K19" s="57" t="n"/>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="44" t="inlineStr">
+      <c r="A20" s="58" t="inlineStr">
         <is>
           <t>Sep '26</t>
         </is>
       </c>
-      <c r="B20" s="45" t="n"/>
-      <c r="C20" s="45" t="n"/>
-      <c r="D20" s="45" t="n"/>
-      <c r="E20" s="45" t="n"/>
-      <c r="F20" s="46">
+      <c r="B20" s="59" t="n"/>
+      <c r="C20" s="59" t="n"/>
+      <c r="D20" s="59" t="n"/>
+      <c r="E20" s="59" t="n"/>
+      <c r="F20" s="60">
         <f>IFERROR(SUM(B20:E20),"")</f>
         <v/>
       </c>
-      <c r="G20" s="47" t="n">
+      <c r="G20" s="61" t="n">
         <v>630</v>
       </c>
-      <c r="H20" s="48">
+      <c r="H20" s="62">
         <f>IFERROR(G20-F20,"")</f>
         <v/>
       </c>
-      <c r="I20" s="45">
+      <c r="I20" s="59">
         <f>IFERROR(MAX(0,MIN(167.63,I19+H20)),"")</f>
         <v/>
       </c>
-      <c r="J20" s="49">
+      <c r="J20" s="63">
         <f>IFERROR(MAX(0,H20-MAX(0,167.63-167.63)),"")</f>
         <v/>
       </c>
       <c r="K20" s="2" t="n"/>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="37" t="inlineStr">
+      <c r="A21" s="51" t="inlineStr">
         <is>
           <t>Oct '26</t>
         </is>
       </c>
-      <c r="B21" s="38" t="n"/>
-      <c r="C21" s="38" t="n"/>
-      <c r="D21" s="38" t="n"/>
-      <c r="E21" s="38" t="n"/>
-      <c r="F21" s="39">
+      <c r="B21" s="52" t="n"/>
+      <c r="C21" s="52" t="n"/>
+      <c r="D21" s="52" t="n"/>
+      <c r="E21" s="52" t="n"/>
+      <c r="F21" s="53">
         <f>IFERROR(SUM(B21:E21),"")</f>
         <v/>
       </c>
-      <c r="G21" s="40" t="n">
+      <c r="G21" s="54" t="n">
         <v>630</v>
       </c>
-      <c r="H21" s="41">
+      <c r="H21" s="55">
         <f>IFERROR(G21-F21,"")</f>
         <v/>
       </c>
-      <c r="I21" s="38">
+      <c r="I21" s="52">
         <f>IFERROR(MAX(0,MIN(167.63,I20+H21)),"")</f>
         <v/>
       </c>
-      <c r="J21" s="42">
+      <c r="J21" s="56">
         <f>IFERROR(MAX(0,H21-MAX(0,167.63-167.63)),"")</f>
         <v/>
       </c>
-      <c r="K21" s="43" t="n"/>
+      <c r="K21" s="57" t="n"/>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="44" t="inlineStr">
+      <c r="A22" s="58" t="inlineStr">
         <is>
           <t>Nov '26</t>
         </is>
       </c>
-      <c r="B22" s="45" t="n"/>
-      <c r="C22" s="45" t="n"/>
-      <c r="D22" s="45" t="n"/>
-      <c r="E22" s="45" t="n"/>
-      <c r="F22" s="46">
+      <c r="B22" s="59" t="n"/>
+      <c r="C22" s="59" t="n"/>
+      <c r="D22" s="59" t="n"/>
+      <c r="E22" s="59" t="n"/>
+      <c r="F22" s="60">
         <f>IFERROR(SUM(B22:E22),"")</f>
         <v/>
       </c>
-      <c r="G22" s="47" t="n">
+      <c r="G22" s="61" t="n">
         <v>630</v>
       </c>
-      <c r="H22" s="48">
+      <c r="H22" s="62">
         <f>IFERROR(G22-F22,"")</f>
         <v/>
       </c>
-      <c r="I22" s="45">
+      <c r="I22" s="59">
         <f>IFERROR(MAX(0,MIN(167.63,I21+H22)),"")</f>
         <v/>
       </c>
-      <c r="J22" s="49">
+      <c r="J22" s="63">
         <f>IFERROR(MAX(0,H22-MAX(0,167.63-167.63)),"")</f>
         <v/>
       </c>
       <c r="K22" s="2" t="n"/>
     </row>
     <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="37" t="inlineStr">
+      <c r="A23" s="51" t="inlineStr">
         <is>
           <t>Dec '26</t>
         </is>
       </c>
-      <c r="B23" s="38" t="n"/>
-      <c r="C23" s="38" t="n"/>
-      <c r="D23" s="38" t="n"/>
-      <c r="E23" s="38" t="n"/>
-      <c r="F23" s="39">
+      <c r="B23" s="52" t="n"/>
+      <c r="C23" s="52" t="n"/>
+      <c r="D23" s="52" t="n"/>
+      <c r="E23" s="52" t="n"/>
+      <c r="F23" s="53">
         <f>IFERROR(SUM(B23:E23),"")</f>
         <v/>
       </c>
-      <c r="G23" s="40" t="n">
+      <c r="G23" s="54" t="n">
         <v>630</v>
       </c>
-      <c r="H23" s="41">
+      <c r="H23" s="55">
         <f>IFERROR(G23-F23,"")</f>
         <v/>
       </c>
-      <c r="I23" s="38">
+      <c r="I23" s="52">
         <f>IFERROR(MAX(0,MIN(167.63,I22+H23)),"")</f>
         <v/>
       </c>
-      <c r="J23" s="42">
+      <c r="J23" s="56">
         <f>IFERROR(MAX(0,H23-MAX(0,167.63-167.63)),"")</f>
         <v/>
       </c>
-      <c r="K23" s="43" t="n"/>
+      <c r="K23" s="57" t="n"/>
     </row>
     <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="44" t="inlineStr">
+      <c r="A24" s="58" t="inlineStr">
         <is>
           <t>Jan '27</t>
         </is>
       </c>
-      <c r="B24" s="45" t="n"/>
-      <c r="C24" s="45" t="n"/>
-      <c r="D24" s="45" t="n"/>
-      <c r="E24" s="45" t="n"/>
-      <c r="F24" s="46">
+      <c r="B24" s="59" t="n"/>
+      <c r="C24" s="59" t="n"/>
+      <c r="D24" s="59" t="n"/>
+      <c r="E24" s="59" t="n"/>
+      <c r="F24" s="60">
         <f>IFERROR(SUM(B24:E24),"")</f>
         <v/>
       </c>
-      <c r="G24" s="47" t="n">
+      <c r="G24" s="61" t="n">
         <v>630</v>
       </c>
-      <c r="H24" s="48">
+      <c r="H24" s="62">
         <f>IFERROR(G24-F24,"")</f>
         <v/>
       </c>
-      <c r="I24" s="45">
+      <c r="I24" s="59">
         <f>IFERROR(MAX(0,MIN(167.63,I23+H24)),"")</f>
         <v/>
       </c>
-      <c r="J24" s="49">
+      <c r="J24" s="63">
         <f>IFERROR(MAX(0,H24-MAX(0,167.63-167.63)),"")</f>
         <v/>
       </c>
       <c r="K24" s="2" t="n"/>
     </row>
     <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="37" t="inlineStr">
+      <c r="A25" s="51" t="inlineStr">
         <is>
           <t>Feb '27</t>
         </is>
       </c>
-      <c r="B25" s="38" t="n"/>
-      <c r="C25" s="38" t="n"/>
-      <c r="D25" s="38" t="n"/>
-      <c r="E25" s="38" t="n"/>
-      <c r="F25" s="39">
+      <c r="B25" s="52" t="n"/>
+      <c r="C25" s="52" t="n"/>
+      <c r="D25" s="52" t="n"/>
+      <c r="E25" s="52" t="n"/>
+      <c r="F25" s="53">
         <f>IFERROR(SUM(B25:E25),"")</f>
         <v/>
       </c>
-      <c r="G25" s="40" t="n">
+      <c r="G25" s="54" t="n">
         <v>630</v>
       </c>
-      <c r="H25" s="41">
+      <c r="H25" s="55">
         <f>IFERROR(G25-F25,"")</f>
         <v/>
       </c>
-      <c r="I25" s="38">
+      <c r="I25" s="52">
         <f>IFERROR(MAX(0,MIN(167.63,I24+H25)),"")</f>
         <v/>
       </c>
-      <c r="J25" s="42">
+      <c r="J25" s="56">
         <f>IFERROR(MAX(0,H25-MAX(0,167.63-167.63)),"")</f>
         <v/>
       </c>
-      <c r="K25" s="43" t="n"/>
+      <c r="K25" s="57" t="n"/>
     </row>
     <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="44" t="inlineStr">
+      <c r="A26" s="58" t="inlineStr">
         <is>
           <t>Mar '27</t>
         </is>
       </c>
-      <c r="B26" s="45" t="n"/>
-      <c r="C26" s="45" t="n"/>
-      <c r="D26" s="45" t="n"/>
-      <c r="E26" s="45" t="n"/>
-      <c r="F26" s="46">
+      <c r="B26" s="59" t="n"/>
+      <c r="C26" s="59" t="n"/>
+      <c r="D26" s="59" t="n"/>
+      <c r="E26" s="59" t="n"/>
+      <c r="F26" s="60">
         <f>IFERROR(SUM(B26:E26),"")</f>
         <v/>
       </c>
-      <c r="G26" s="47" t="n">
+      <c r="G26" s="61" t="n">
         <v>630</v>
       </c>
-      <c r="H26" s="48">
+      <c r="H26" s="62">
         <f>IFERROR(G26-F26,"")</f>
         <v/>
       </c>
-      <c r="I26" s="45">
+      <c r="I26" s="59">
         <f>IFERROR(MAX(0,MIN(167.63,I25+H26)),"")</f>
         <v/>
       </c>
-      <c r="J26" s="49">
+      <c r="J26" s="63">
         <f>IFERROR(MAX(0,H26-MAX(0,167.63-167.63)),"")</f>
         <v/>
       </c>
       <c r="K26" s="2" t="n"/>
     </row>
     <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="37" t="inlineStr">
+      <c r="A27" s="51" t="inlineStr">
         <is>
           <t>Apr '27</t>
         </is>
       </c>
-      <c r="B27" s="38" t="n"/>
-      <c r="C27" s="38" t="n"/>
-      <c r="D27" s="38" t="n"/>
-      <c r="E27" s="38" t="n"/>
-      <c r="F27" s="39">
+      <c r="B27" s="52" t="n"/>
+      <c r="C27" s="52" t="n"/>
+      <c r="D27" s="52" t="n"/>
+      <c r="E27" s="52" t="n"/>
+      <c r="F27" s="53">
         <f>IFERROR(SUM(B27:E27),"")</f>
         <v/>
       </c>
-      <c r="G27" s="40" t="n">
+      <c r="G27" s="54" t="n">
         <v>630</v>
       </c>
-      <c r="H27" s="41">
+      <c r="H27" s="55">
         <f>IFERROR(G27-F27,"")</f>
         <v/>
       </c>
-      <c r="I27" s="38">
+      <c r="I27" s="52">
         <f>IFERROR(MAX(0,MIN(167.63,I26+H27)),"")</f>
         <v/>
       </c>
-      <c r="J27" s="42">
+      <c r="J27" s="56">
         <f>IFERROR(MAX(0,H27-MAX(0,167.63-167.63)),"")</f>
         <v/>
       </c>
-      <c r="K27" s="43" t="n"/>
+      <c r="K27" s="57" t="n"/>
     </row>
     <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="44" t="inlineStr">
+      <c r="A28" s="58" t="inlineStr">
         <is>
           <t>May '27</t>
         </is>
       </c>
-      <c r="B28" s="45" t="n"/>
-      <c r="C28" s="45" t="n"/>
-      <c r="D28" s="45" t="n"/>
-      <c r="E28" s="45" t="n"/>
-      <c r="F28" s="46">
+      <c r="B28" s="59" t="n"/>
+      <c r="C28" s="59" t="n"/>
+      <c r="D28" s="59" t="n"/>
+      <c r="E28" s="59" t="n"/>
+      <c r="F28" s="60">
         <f>IFERROR(SUM(B28:E28),"")</f>
         <v/>
       </c>
-      <c r="G28" s="47" t="n">
+      <c r="G28" s="61" t="n">
         <v>630</v>
       </c>
-      <c r="H28" s="48">
+      <c r="H28" s="62">
         <f>IFERROR(G28-F28,"")</f>
         <v/>
       </c>
-      <c r="I28" s="45">
+      <c r="I28" s="59">
         <f>IFERROR(MAX(0,MIN(167.63,I27+H28)),"")</f>
         <v/>
       </c>
-      <c r="J28" s="49">
+      <c r="J28" s="63">
         <f>IFERROR(MAX(0,H28-MAX(0,167.63-167.63)),"")</f>
         <v/>
       </c>
       <c r="K28" s="2" t="n"/>
     </row>
     <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="37" t="inlineStr">
+      <c r="A29" s="51" t="inlineStr">
         <is>
           <t>Jun '27</t>
         </is>
       </c>
-      <c r="B29" s="38" t="n"/>
-      <c r="C29" s="38" t="n"/>
-      <c r="D29" s="38" t="n"/>
-      <c r="E29" s="38" t="n"/>
-      <c r="F29" s="39">
+      <c r="B29" s="52" t="n"/>
+      <c r="C29" s="52" t="n"/>
+      <c r="D29" s="52" t="n"/>
+      <c r="E29" s="52" t="n"/>
+      <c r="F29" s="53">
         <f>IFERROR(SUM(B29:E29),"")</f>
         <v/>
       </c>
-      <c r="G29" s="40" t="n">
+      <c r="G29" s="54" t="n">
         <v>630</v>
       </c>
-      <c r="H29" s="41">
+      <c r="H29" s="55">
         <f>IFERROR(G29-F29,"")</f>
         <v/>
       </c>
-      <c r="I29" s="38">
+      <c r="I29" s="52">
         <f>IFERROR(MAX(0,MIN(167.63,I28+H29)),"")</f>
         <v/>
       </c>
-      <c r="J29" s="42">
+      <c r="J29" s="56">
         <f>IFERROR(MAX(0,H29-MAX(0,167.63-167.63)),"")</f>
         <v/>
       </c>
-      <c r="K29" s="43" t="n"/>
+      <c r="K29" s="57" t="n"/>
     </row>
     <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="44" t="inlineStr">
+      <c r="A30" s="58" t="inlineStr">
         <is>
           <t>Jul '27</t>
         </is>
       </c>
-      <c r="B30" s="45" t="n"/>
-      <c r="C30" s="45" t="n"/>
-      <c r="D30" s="45" t="n"/>
-      <c r="E30" s="45" t="n"/>
-      <c r="F30" s="46">
+      <c r="B30" s="59" t="n"/>
+      <c r="C30" s="59" t="n"/>
+      <c r="D30" s="59" t="n"/>
+      <c r="E30" s="59" t="n"/>
+      <c r="F30" s="60">
         <f>IFERROR(SUM(B30:E30),"")</f>
         <v/>
       </c>
-      <c r="G30" s="47" t="n">
+      <c r="G30" s="61" t="n">
         <v>630</v>
       </c>
-      <c r="H30" s="48">
+      <c r="H30" s="62">
         <f>IFERROR(G30-F30,"")</f>
         <v/>
       </c>
-      <c r="I30" s="45">
+      <c r="I30" s="59">
         <f>IFERROR(MAX(0,MIN(167.63,I29+H30)),"")</f>
         <v/>
       </c>
-      <c r="J30" s="49">
+      <c r="J30" s="63">
         <f>IFERROR(MAX(0,H30-MAX(0,167.63-167.63)),"")</f>
         <v/>
       </c>
       <c r="K30" s="2" t="n"/>
     </row>
     <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="37" t="inlineStr">
+      <c r="A31" s="51" t="inlineStr">
         <is>
           <t>Aug '27</t>
         </is>
       </c>
-      <c r="B31" s="38" t="n"/>
-      <c r="C31" s="38" t="n"/>
-      <c r="D31" s="38" t="n"/>
-      <c r="E31" s="38" t="n"/>
-      <c r="F31" s="39">
+      <c r="B31" s="52" t="n"/>
+      <c r="C31" s="52" t="n"/>
+      <c r="D31" s="52" t="n"/>
+      <c r="E31" s="52" t="n"/>
+      <c r="F31" s="53">
         <f>IFERROR(SUM(B31:E31),"")</f>
         <v/>
       </c>
-      <c r="G31" s="40" t="n">
+      <c r="G31" s="54" t="n">
         <v>630</v>
       </c>
-      <c r="H31" s="41">
+      <c r="H31" s="55">
         <f>IFERROR(G31-F31,"")</f>
         <v/>
       </c>
-      <c r="I31" s="38">
+      <c r="I31" s="52">
         <f>IFERROR(MAX(0,MIN(167.63,I30+H31)),"")</f>
         <v/>
       </c>
-      <c r="J31" s="42">
+      <c r="J31" s="56">
         <f>IFERROR(MAX(0,H31-MAX(0,167.63-167.63)),"")</f>
         <v/>
       </c>
-      <c r="K31" s="43" t="n"/>
+      <c r="K31" s="57" t="n"/>
     </row>
     <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="44" t="inlineStr">
+      <c r="A32" s="58" t="inlineStr">
         <is>
           <t>Sep '27</t>
         </is>
       </c>
-      <c r="B32" s="45" t="n"/>
-      <c r="C32" s="45" t="n"/>
-      <c r="D32" s="45" t="n"/>
-      <c r="E32" s="45" t="n"/>
-      <c r="F32" s="46">
+      <c r="B32" s="59" t="n"/>
+      <c r="C32" s="59" t="n"/>
+      <c r="D32" s="59" t="n"/>
+      <c r="E32" s="59" t="n"/>
+      <c r="F32" s="60">
         <f>IFERROR(SUM(B32:E32),"")</f>
         <v/>
       </c>
-      <c r="G32" s="47" t="n">
+      <c r="G32" s="61" t="n">
         <v>630</v>
       </c>
-      <c r="H32" s="48">
+      <c r="H32" s="62">
         <f>IFERROR(G32-F32,"")</f>
         <v/>
       </c>
-      <c r="I32" s="45">
+      <c r="I32" s="59">
         <f>IFERROR(MAX(0,MIN(167.63,I31+H32)),"")</f>
         <v/>
       </c>
-      <c r="J32" s="49">
+      <c r="J32" s="63">
         <f>IFERROR(MAX(0,H32-MAX(0,167.63-167.63)),"")</f>
         <v/>
       </c>
       <c r="K32" s="2" t="n"/>
     </row>
     <row r="33" ht="20" customHeight="1">
-      <c r="A33" s="37" t="inlineStr">
+      <c r="A33" s="51" t="inlineStr">
         <is>
           <t>Oct '27</t>
         </is>
       </c>
-      <c r="B33" s="38" t="n"/>
-      <c r="C33" s="38" t="n"/>
-      <c r="D33" s="38" t="n"/>
-      <c r="E33" s="38" t="n"/>
-      <c r="F33" s="39">
+      <c r="B33" s="52" t="n"/>
+      <c r="C33" s="52" t="n"/>
+      <c r="D33" s="52" t="n"/>
+      <c r="E33" s="52" t="n"/>
+      <c r="F33" s="53">
         <f>IFERROR(SUM(B33:E33),"")</f>
         <v/>
       </c>
-      <c r="G33" s="40" t="n">
+      <c r="G33" s="54" t="n">
         <v>630</v>
       </c>
-      <c r="H33" s="41">
+      <c r="H33" s="55">
         <f>IFERROR(G33-F33,"")</f>
         <v/>
       </c>
-      <c r="I33" s="38">
+      <c r="I33" s="52">
         <f>IFERROR(MAX(0,MIN(167.63,I32+H33)),"")</f>
         <v/>
       </c>
-      <c r="J33" s="42">
+      <c r="J33" s="56">
         <f>IFERROR(MAX(0,H33-MAX(0,167.63-167.63)),"")</f>
         <v/>
       </c>
-      <c r="K33" s="43" t="n"/>
+      <c r="K33" s="57" t="n"/>
     </row>
     <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="44" t="inlineStr">
+      <c r="A34" s="58" t="inlineStr">
         <is>
           <t>Nov '27</t>
         </is>
       </c>
-      <c r="B34" s="45" t="n"/>
-      <c r="C34" s="45" t="n"/>
-      <c r="D34" s="45" t="n"/>
-      <c r="E34" s="45" t="n"/>
-      <c r="F34" s="46">
+      <c r="B34" s="59" t="n"/>
+      <c r="C34" s="59" t="n"/>
+      <c r="D34" s="59" t="n"/>
+      <c r="E34" s="59" t="n"/>
+      <c r="F34" s="60">
         <f>IFERROR(SUM(B34:E34),"")</f>
         <v/>
       </c>
-      <c r="G34" s="47" t="n">
+      <c r="G34" s="61" t="n">
         <v>630</v>
       </c>
-      <c r="H34" s="48">
+      <c r="H34" s="62">
         <f>IFERROR(G34-F34,"")</f>
         <v/>
       </c>
-      <c r="I34" s="45">
+      <c r="I34" s="59">
         <f>IFERROR(MAX(0,MIN(167.63,I33+H34)),"")</f>
         <v/>
       </c>
-      <c r="J34" s="49">
+      <c r="J34" s="63">
         <f>IFERROR(MAX(0,H34-MAX(0,167.63-167.63)),"")</f>
         <v/>
       </c>
       <c r="K34" s="2" t="n"/>
     </row>
     <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="37" t="inlineStr">
+      <c r="A35" s="51" t="inlineStr">
         <is>
           <t>Dec '27</t>
         </is>
       </c>
-      <c r="B35" s="38" t="n"/>
-      <c r="C35" s="38" t="n"/>
-      <c r="D35" s="38" t="n"/>
-      <c r="E35" s="38" t="n"/>
-      <c r="F35" s="39">
+      <c r="B35" s="52" t="n"/>
+      <c r="C35" s="52" t="n"/>
+      <c r="D35" s="52" t="n"/>
+      <c r="E35" s="52" t="n"/>
+      <c r="F35" s="53">
         <f>IFERROR(SUM(B35:E35),"")</f>
         <v/>
       </c>
-      <c r="G35" s="40" t="n">
+      <c r="G35" s="54" t="n">
         <v>630</v>
       </c>
-      <c r="H35" s="41">
+      <c r="H35" s="55">
         <f>IFERROR(G35-F35,"")</f>
         <v/>
       </c>
-      <c r="I35" s="38">
+      <c r="I35" s="52">
         <f>IFERROR(MAX(0,MIN(167.63,I34+H35)),"")</f>
         <v/>
       </c>
-      <c r="J35" s="42">
+      <c r="J35" s="56">
         <f>IFERROR(MAX(0,H35-MAX(0,167.63-167.63)),"")</f>
         <v/>
       </c>
-      <c r="K35" s="43" t="n"/>
+      <c r="K35" s="57" t="n"/>
     </row>
     <row r="37" ht="24" customHeight="1">
-      <c r="A37" s="50" t="inlineStr">
+      <c r="A37" s="64" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B37" s="51">
+      <c r="B37" s="65">
         <f>SUM(B5:B17)</f>
         <v/>
       </c>
-      <c r="C37" s="51">
+      <c r="C37" s="65">
         <f>SUM(C5:C17)</f>
         <v/>
       </c>
-      <c r="D37" s="51">
+      <c r="D37" s="65">
         <f>SUM(D5:D17)</f>
         <v/>
       </c>
-      <c r="E37" s="51">
+      <c r="E37" s="65">
         <f>SUM(E5:E17)</f>
         <v/>
       </c>
-      <c r="F37" s="51">
+      <c r="F37" s="65">
         <f>SUM(F5:F17)</f>
         <v/>
       </c>
-      <c r="G37" s="51">
+      <c r="G37" s="65">
         <f>630*13</f>
         <v/>
       </c>
-      <c r="H37" s="51">
+      <c r="H37" s="65">
         <f>SUM(H5:H17)</f>
         <v/>
       </c>
-      <c r="J37" s="51">
+      <c r="J37" s="65">
         <f>SUM(J5:J17)</f>
         <v/>
       </c>
     </row>
     <row r="38" ht="20" customHeight="1">
-      <c r="A38" s="44" t="inlineStr">
+      <c r="A38" s="58" t="inlineStr">
         <is>
           <t>AVERAGES</t>
         </is>
       </c>
-      <c r="B38" s="45">
+      <c r="B38" s="59">
         <f>IFERROR(B37/COUNTA(B5:B17),"")</f>
         <v/>
       </c>
-      <c r="C38" s="45">
+      <c r="C38" s="59">
         <f>IFERROR(C37/COUNTA(C5:C17),"")</f>
         <v/>
       </c>
-      <c r="D38" s="45">
+      <c r="D38" s="59">
         <f>IFERROR(D37/COUNTA(D5:D17),"")</f>
         <v/>
       </c>
-      <c r="E38" s="45">
+      <c r="E38" s="59">
         <f>IFERROR(E37/COUNTA(E5:E17),"")</f>
         <v/>
       </c>
-      <c r="F38" s="45">
+      <c r="F38" s="59">
         <f>IFERROR(F37/COUNTA(F5:F17),"")</f>
         <v/>
       </c>
-      <c r="H38" s="45">
+      <c r="H38" s="59">
         <f>IFERROR(H37/COUNTA(H5:H17),"")</f>
         <v/>
       </c>
@@ -2677,1078 +3154,1078 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="52" t="inlineStr">
+      <c r="A1" s="66" t="inlineStr">
         <is>
           <t>PER UTILITY — Actuals vs Targets</t>
         </is>
       </c>
     </row>
     <row r="3" ht="26" customHeight="1">
-      <c r="A3" s="53" t="inlineStr">
+      <c r="A3" s="67" t="inlineStr">
         <is>
           <t>WATER  ·  fund $90/mo  ·  avg $49  ·  cushion $41/mo</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="44" t="inlineStr">
+      <c r="A4" s="58" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B4" s="44" t="inlineStr">
+      <c r="B4" s="58" t="inlineStr">
         <is>
           <t>Actual</t>
         </is>
       </c>
-      <c r="C4" s="44" t="inlineStr">
+      <c r="C4" s="58" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="D4" s="44" t="inlineStr">
+      <c r="D4" s="58" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="E4" s="44" t="inlineStr">
+      <c r="E4" s="58" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="54" t="inlineStr">
+      <c r="A5" s="68" t="inlineStr">
         <is>
           <t>Jun '25</t>
         </is>
       </c>
-      <c r="B5" s="38" t="n">
+      <c r="B5" s="52" t="n">
         <v>22.5</v>
       </c>
-      <c r="C5" s="55" t="n">
+      <c r="C5" s="69" t="n">
         <v>90</v>
       </c>
-      <c r="D5" s="56">
+      <c r="D5" s="70">
         <f>IFERROR(C5-B5,"")</f>
         <v/>
       </c>
-      <c r="E5" s="43" t="n"/>
+      <c r="E5" s="57" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="57" t="inlineStr">
+      <c r="A6" s="71" t="inlineStr">
         <is>
           <t>Jul '25</t>
         </is>
       </c>
-      <c r="B6" s="45" t="n">
+      <c r="B6" s="59" t="n">
         <v>28.32</v>
       </c>
-      <c r="C6" s="58" t="n">
+      <c r="C6" s="72" t="n">
         <v>90</v>
       </c>
-      <c r="D6" s="59">
+      <c r="D6" s="73">
         <f>IFERROR(C6-B6,"")</f>
         <v/>
       </c>
       <c r="E6" s="2" t="n"/>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="54" t="inlineStr">
+      <c r="A7" s="68" t="inlineStr">
         <is>
           <t>Aug '25</t>
         </is>
       </c>
-      <c r="B7" s="38" t="n">
+      <c r="B7" s="52" t="n">
         <v>24.35</v>
       </c>
-      <c r="C7" s="55" t="n">
+      <c r="C7" s="69" t="n">
         <v>90</v>
       </c>
-      <c r="D7" s="56">
+      <c r="D7" s="70">
         <f>IFERROR(C7-B7,"")</f>
         <v/>
       </c>
-      <c r="E7" s="43" t="n"/>
+      <c r="E7" s="57" t="n"/>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="57" t="inlineStr">
+      <c r="A8" s="71" t="inlineStr">
         <is>
           <t>Sep '25</t>
         </is>
       </c>
-      <c r="B8" s="45" t="n">
+      <c r="B8" s="59" t="n">
         <v>33.54</v>
       </c>
-      <c r="C8" s="58" t="n">
+      <c r="C8" s="72" t="n">
         <v>90</v>
       </c>
-      <c r="D8" s="59">
+      <c r="D8" s="73">
         <f>IFERROR(C8-B8,"")</f>
         <v/>
       </c>
       <c r="E8" s="2" t="n"/>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="54" t="inlineStr">
+      <c r="A9" s="68" t="inlineStr">
         <is>
           <t>Oct '25</t>
         </is>
       </c>
-      <c r="B9" s="38" t="n">
+      <c r="B9" s="52" t="n">
         <v>35.97</v>
       </c>
-      <c r="C9" s="55" t="n">
+      <c r="C9" s="69" t="n">
         <v>90</v>
       </c>
-      <c r="D9" s="56">
+      <c r="D9" s="70">
         <f>IFERROR(C9-B9,"")</f>
         <v/>
       </c>
-      <c r="E9" s="43" t="n"/>
+      <c r="E9" s="57" t="n"/>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="57" t="inlineStr">
+      <c r="A10" s="71" t="inlineStr">
         <is>
           <t>Nov '25</t>
         </is>
       </c>
-      <c r="B10" s="45" t="n">
+      <c r="B10" s="59" t="n">
         <v>35.97</v>
       </c>
-      <c r="C10" s="58" t="n">
+      <c r="C10" s="72" t="n">
         <v>90</v>
       </c>
-      <c r="D10" s="59">
+      <c r="D10" s="73">
         <f>IFERROR(C10-B10,"")</f>
         <v/>
       </c>
       <c r="E10" s="2" t="n"/>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="54" t="inlineStr">
+      <c r="A11" s="68" t="inlineStr">
         <is>
           <t>Dec '25</t>
         </is>
       </c>
-      <c r="B11" s="38" t="n">
+      <c r="B11" s="52" t="n">
         <v>44.13</v>
       </c>
-      <c r="C11" s="55" t="n">
+      <c r="C11" s="69" t="n">
         <v>90</v>
       </c>
-      <c r="D11" s="56">
+      <c r="D11" s="70">
         <f>IFERROR(C11-B11,"")</f>
         <v/>
       </c>
-      <c r="E11" s="43" t="n"/>
+      <c r="E11" s="57" t="n"/>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="57" t="inlineStr">
+      <c r="A12" s="71" t="inlineStr">
         <is>
           <t>Jan '26</t>
         </is>
       </c>
-      <c r="B12" s="45" t="n">
+      <c r="B12" s="59" t="n">
         <v>40.52</v>
       </c>
-      <c r="C12" s="58" t="n">
+      <c r="C12" s="72" t="n">
         <v>90</v>
       </c>
-      <c r="D12" s="59">
+      <c r="D12" s="73">
         <f>IFERROR(C12-B12,"")</f>
         <v/>
       </c>
       <c r="E12" s="2" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="54" t="inlineStr">
+      <c r="A13" s="68" t="inlineStr">
         <is>
           <t>Feb '26</t>
         </is>
       </c>
-      <c r="B13" s="38" t="n">
+      <c r="B13" s="52" t="n">
         <v>31.02</v>
       </c>
-      <c r="C13" s="55" t="n">
+      <c r="C13" s="69" t="n">
         <v>90</v>
       </c>
-      <c r="D13" s="56">
+      <c r="D13" s="70">
         <f>IFERROR(C13-B13,"")</f>
         <v/>
       </c>
-      <c r="E13" s="43" t="n"/>
+      <c r="E13" s="57" t="n"/>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="57" t="inlineStr">
+      <c r="A14" s="71" t="inlineStr">
         <is>
           <t>Mar '26</t>
         </is>
       </c>
-      <c r="B14" s="45" t="n">
+      <c r="B14" s="59" t="n">
         <v>39.61</v>
       </c>
-      <c r="C14" s="58" t="n">
+      <c r="C14" s="72" t="n">
         <v>90</v>
       </c>
-      <c r="D14" s="59">
+      <c r="D14" s="73">
         <f>IFERROR(C14-B14,"")</f>
         <v/>
       </c>
       <c r="E14" s="2" t="n"/>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="54" t="inlineStr">
+      <c r="A15" s="68" t="inlineStr">
         <is>
           <t>Apr '26</t>
         </is>
       </c>
-      <c r="B15" s="38" t="n">
+      <c r="B15" s="52" t="n">
         <v>86.5</v>
       </c>
-      <c r="C15" s="55" t="n">
+      <c r="C15" s="69" t="n">
         <v>90</v>
       </c>
-      <c r="D15" s="56">
+      <c r="D15" s="70">
         <f>IFERROR(C15-B15,"")</f>
         <v/>
       </c>
-      <c r="E15" s="43" t="n"/>
+      <c r="E15" s="57" t="n"/>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="57" t="inlineStr">
+      <c r="A16" s="71" t="inlineStr">
         <is>
           <t>Jun '26</t>
         </is>
       </c>
-      <c r="B16" s="45" t="n">
+      <c r="B16" s="59" t="n">
         <v>166.96</v>
       </c>
-      <c r="C16" s="58" t="n">
+      <c r="C16" s="72" t="n">
         <v>90</v>
       </c>
-      <c r="D16" s="59">
+      <c r="D16" s="73">
         <f>IFERROR(C16-B16,"")</f>
         <v/>
       </c>
       <c r="E16" s="2" t="n"/>
     </row>
     <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="60" t="inlineStr">
+      <c r="A17" s="74" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B17" s="61">
+      <c r="B17" s="75">
         <f>SUM(B5:B16)</f>
         <v/>
       </c>
-      <c r="C17" s="61" t="n">
+      <c r="C17" s="75" t="n">
         <v>1080</v>
       </c>
-      <c r="D17" s="62">
+      <c r="D17" s="76">
         <f>C17-B17</f>
         <v/>
       </c>
     </row>
     <row r="20" ht="26" customHeight="1">
-      <c r="A20" s="63" t="inlineStr">
+      <c r="A20" s="77" t="inlineStr">
         <is>
           <t>POWER  ·  fund $453/mo  ·  avg $344  ·  cushion $109/mo</t>
         </is>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="44" t="inlineStr">
+      <c r="A21" s="58" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B21" s="44" t="inlineStr">
+      <c r="B21" s="58" t="inlineStr">
         <is>
           <t>Actual</t>
         </is>
       </c>
-      <c r="C21" s="44" t="inlineStr">
+      <c r="C21" s="58" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="D21" s="44" t="inlineStr">
+      <c r="D21" s="58" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="E21" s="44" t="inlineStr">
+      <c r="E21" s="58" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="54" t="inlineStr">
+      <c r="A22" s="68" t="inlineStr">
         <is>
           <t>Jun '25</t>
         </is>
       </c>
-      <c r="B22" s="38" t="n">
+      <c r="B22" s="52" t="n">
         <v>368.62</v>
       </c>
-      <c r="C22" s="55" t="n">
+      <c r="C22" s="69" t="n">
         <v>453</v>
       </c>
-      <c r="D22" s="56">
+      <c r="D22" s="70">
         <f>IFERROR(C22-B22,"")</f>
         <v/>
       </c>
-      <c r="E22" s="43" t="n"/>
+      <c r="E22" s="57" t="n"/>
     </row>
     <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="57" t="inlineStr">
+      <c r="A23" s="71" t="inlineStr">
         <is>
           <t>Jul '25</t>
         </is>
       </c>
-      <c r="B23" s="45" t="n">
+      <c r="B23" s="59" t="n">
         <v>440.17</v>
       </c>
-      <c r="C23" s="58" t="n">
+      <c r="C23" s="72" t="n">
         <v>453</v>
       </c>
-      <c r="D23" s="59">
+      <c r="D23" s="73">
         <f>IFERROR(C23-B23,"")</f>
         <v/>
       </c>
       <c r="E23" s="2" t="n"/>
     </row>
     <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="54" t="inlineStr">
+      <c r="A24" s="68" t="inlineStr">
         <is>
           <t>Aug '25</t>
         </is>
       </c>
-      <c r="B24" s="38" t="n">
+      <c r="B24" s="52" t="n">
         <v>429.27</v>
       </c>
-      <c r="C24" s="55" t="n">
+      <c r="C24" s="69" t="n">
         <v>453</v>
       </c>
-      <c r="D24" s="56">
+      <c r="D24" s="70">
         <f>IFERROR(C24-B24,"")</f>
         <v/>
       </c>
-      <c r="E24" s="43" t="n"/>
+      <c r="E24" s="57" t="n"/>
     </row>
     <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="57" t="inlineStr">
+      <c r="A25" s="71" t="inlineStr">
         <is>
           <t>Sep '25</t>
         </is>
       </c>
-      <c r="B25" s="45" t="n">
+      <c r="B25" s="59" t="n">
         <v>381.57</v>
       </c>
-      <c r="C25" s="58" t="n">
+      <c r="C25" s="72" t="n">
         <v>453</v>
       </c>
-      <c r="D25" s="59">
+      <c r="D25" s="73">
         <f>IFERROR(C25-B25,"")</f>
         <v/>
       </c>
       <c r="E25" s="2" t="n"/>
     </row>
     <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="54" t="inlineStr">
+      <c r="A26" s="68" t="inlineStr">
         <is>
           <t>Oct '25</t>
         </is>
       </c>
-      <c r="B26" s="38" t="n">
+      <c r="B26" s="52" t="n">
         <v>248.35</v>
       </c>
-      <c r="C26" s="55" t="n">
+      <c r="C26" s="69" t="n">
         <v>453</v>
       </c>
-      <c r="D26" s="56">
+      <c r="D26" s="70">
         <f>IFERROR(C26-B26,"")</f>
         <v/>
       </c>
-      <c r="E26" s="43" t="n"/>
+      <c r="E26" s="57" t="n"/>
     </row>
     <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="57" t="inlineStr">
+      <c r="A27" s="71" t="inlineStr">
         <is>
           <t>Nov '25</t>
         </is>
       </c>
-      <c r="B27" s="45" t="n">
+      <c r="B27" s="59" t="n">
         <v>264.5</v>
       </c>
-      <c r="C27" s="58" t="n">
+      <c r="C27" s="72" t="n">
         <v>453</v>
       </c>
-      <c r="D27" s="59">
+      <c r="D27" s="73">
         <f>IFERROR(C27-B27,"")</f>
         <v/>
       </c>
       <c r="E27" s="2" t="n"/>
     </row>
     <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="54" t="inlineStr">
+      <c r="A28" s="68" t="inlineStr">
         <is>
           <t>Dec '25</t>
         </is>
       </c>
-      <c r="B28" s="38" t="n">
+      <c r="B28" s="52" t="n">
         <v>415.04</v>
       </c>
-      <c r="C28" s="55" t="n">
+      <c r="C28" s="69" t="n">
         <v>453</v>
       </c>
-      <c r="D28" s="56">
+      <c r="D28" s="70">
         <f>IFERROR(C28-B28,"")</f>
         <v/>
       </c>
-      <c r="E28" s="43" t="n"/>
+      <c r="E28" s="57" t="n"/>
     </row>
     <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="57" t="inlineStr">
+      <c r="A29" s="71" t="inlineStr">
         <is>
           <t>Jan '26</t>
         </is>
       </c>
-      <c r="B29" s="45" t="n">
+      <c r="B29" s="59" t="n">
         <v>541.9</v>
       </c>
-      <c r="C29" s="58" t="n">
+      <c r="C29" s="72" t="n">
         <v>453</v>
       </c>
-      <c r="D29" s="59">
+      <c r="D29" s="73">
         <f>IFERROR(C29-B29,"")</f>
         <v/>
       </c>
       <c r="E29" s="2" t="n"/>
     </row>
     <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="54" t="inlineStr">
+      <c r="A30" s="68" t="inlineStr">
         <is>
           <t>Feb '26</t>
         </is>
       </c>
-      <c r="B30" s="38" t="n">
+      <c r="B30" s="52" t="n">
         <v>388.23</v>
       </c>
-      <c r="C30" s="55" t="n">
+      <c r="C30" s="69" t="n">
         <v>453</v>
       </c>
-      <c r="D30" s="56">
+      <c r="D30" s="70">
         <f>IFERROR(C30-B30,"")</f>
         <v/>
       </c>
-      <c r="E30" s="43" t="n"/>
+      <c r="E30" s="57" t="n"/>
     </row>
     <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="57" t="inlineStr">
+      <c r="A31" s="71" t="inlineStr">
         <is>
           <t>Mar '26</t>
         </is>
       </c>
-      <c r="B31" s="45" t="n">
+      <c r="B31" s="59" t="n">
         <v>226.71</v>
       </c>
-      <c r="C31" s="58" t="n">
+      <c r="C31" s="72" t="n">
         <v>453</v>
       </c>
-      <c r="D31" s="59">
+      <c r="D31" s="73">
         <f>IFERROR(C31-B31,"")</f>
         <v/>
       </c>
       <c r="E31" s="2" t="n"/>
     </row>
     <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="54" t="inlineStr">
+      <c r="A32" s="68" t="inlineStr">
         <is>
           <t>Apr '26</t>
         </is>
       </c>
-      <c r="B32" s="38" t="n">
+      <c r="B32" s="52" t="n">
         <v>206.01</v>
       </c>
-      <c r="C32" s="55" t="n">
+      <c r="C32" s="69" t="n">
         <v>453</v>
       </c>
-      <c r="D32" s="56">
+      <c r="D32" s="70">
         <f>IFERROR(C32-B32,"")</f>
         <v/>
       </c>
-      <c r="E32" s="43" t="n"/>
+      <c r="E32" s="57" t="n"/>
     </row>
     <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="57" t="inlineStr">
+      <c r="A33" s="71" t="inlineStr">
         <is>
           <t>Jun '26</t>
         </is>
       </c>
-      <c r="B33" s="45" t="n">
+      <c r="B33" s="59" t="n">
         <v>220.59</v>
       </c>
-      <c r="C33" s="58" t="n">
+      <c r="C33" s="72" t="n">
         <v>453</v>
       </c>
-      <c r="D33" s="59">
+      <c r="D33" s="73">
         <f>IFERROR(C33-B33,"")</f>
         <v/>
       </c>
       <c r="E33" s="2" t="n"/>
     </row>
     <row r="34" ht="22" customHeight="1">
-      <c r="A34" s="60" t="inlineStr">
+      <c r="A34" s="74" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B34" s="61">
+      <c r="B34" s="75">
         <f>SUM(B22:B33)</f>
         <v/>
       </c>
-      <c r="C34" s="61" t="n">
+      <c r="C34" s="75" t="n">
         <v>5436</v>
       </c>
-      <c r="D34" s="62">
+      <c r="D34" s="76">
         <f>C34-B34</f>
         <v/>
       </c>
     </row>
     <row r="37" ht="26" customHeight="1">
-      <c r="A37" s="64" t="inlineStr">
+      <c r="A37" s="78" t="inlineStr">
         <is>
           <t>INTERNET  ·  fund $64/mo  ·  avg $42  ·  cushion $22/mo</t>
         </is>
       </c>
     </row>
     <row r="38" ht="20" customHeight="1">
-      <c r="A38" s="44" t="inlineStr">
+      <c r="A38" s="58" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B38" s="44" t="inlineStr">
+      <c r="B38" s="58" t="inlineStr">
         <is>
           <t>Actual</t>
         </is>
       </c>
-      <c r="C38" s="44" t="inlineStr">
+      <c r="C38" s="58" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="D38" s="44" t="inlineStr">
+      <c r="D38" s="58" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="E38" s="44" t="inlineStr">
+      <c r="E38" s="58" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="54" t="inlineStr">
+      <c r="A39" s="68" t="inlineStr">
         <is>
           <t>Jun '25</t>
         </is>
       </c>
-      <c r="B39" s="38" t="n">
+      <c r="B39" s="52" t="n">
         <v>42.97</v>
       </c>
-      <c r="C39" s="55" t="n">
+      <c r="C39" s="69" t="n">
         <v>64</v>
       </c>
-      <c r="D39" s="56">
+      <c r="D39" s="70">
         <f>IFERROR(C39-B39,"")</f>
         <v/>
       </c>
-      <c r="E39" s="43" t="n"/>
+      <c r="E39" s="57" t="n"/>
     </row>
     <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="57" t="inlineStr">
+      <c r="A40" s="71" t="inlineStr">
         <is>
           <t>Jul '25</t>
         </is>
       </c>
-      <c r="B40" s="45" t="n">
+      <c r="B40" s="59" t="n">
         <v>42.98</v>
       </c>
-      <c r="C40" s="58" t="n">
+      <c r="C40" s="72" t="n">
         <v>64</v>
       </c>
-      <c r="D40" s="59">
+      <c r="D40" s="73">
         <f>IFERROR(C40-B40,"")</f>
         <v/>
       </c>
       <c r="E40" s="2" t="n"/>
     </row>
     <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="54" t="inlineStr">
+      <c r="A41" s="68" t="inlineStr">
         <is>
           <t>Aug '25</t>
         </is>
       </c>
-      <c r="B41" s="38" t="n">
+      <c r="B41" s="52" t="n">
         <v>42.98</v>
       </c>
-      <c r="C41" s="55" t="n">
+      <c r="C41" s="69" t="n">
         <v>64</v>
       </c>
-      <c r="D41" s="56">
+      <c r="D41" s="70">
         <f>IFERROR(C41-B41,"")</f>
         <v/>
       </c>
-      <c r="E41" s="43" t="n"/>
+      <c r="E41" s="57" t="n"/>
     </row>
     <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="57" t="inlineStr">
+      <c r="A42" s="71" t="inlineStr">
         <is>
           <t>Sep '25</t>
         </is>
       </c>
-      <c r="B42" s="45" t="n">
+      <c r="B42" s="59" t="n">
         <v>63.03</v>
       </c>
-      <c r="C42" s="58" t="n">
+      <c r="C42" s="72" t="n">
         <v>64</v>
       </c>
-      <c r="D42" s="59">
+      <c r="D42" s="73">
         <f>IFERROR(C42-B42,"")</f>
         <v/>
       </c>
       <c r="E42" s="2" t="n"/>
     </row>
     <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="54" t="inlineStr">
+      <c r="A43" s="68" t="inlineStr">
         <is>
           <t>Oct '25</t>
         </is>
       </c>
-      <c r="B43" s="38" t="n">
+      <c r="B43" s="52" t="n">
         <v>63.03</v>
       </c>
-      <c r="C43" s="55" t="n">
+      <c r="C43" s="69" t="n">
         <v>64</v>
       </c>
-      <c r="D43" s="56">
+      <c r="D43" s="70">
         <f>IFERROR(C43-B43,"")</f>
         <v/>
       </c>
-      <c r="E43" s="43" t="n"/>
+      <c r="E43" s="57" t="n"/>
     </row>
     <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="57" t="inlineStr">
+      <c r="A44" s="71" t="inlineStr">
         <is>
           <t>Nov '25</t>
         </is>
       </c>
-      <c r="B44" s="45" t="n">
+      <c r="B44" s="59" t="n">
         <v>63.03</v>
       </c>
-      <c r="C44" s="58" t="n">
+      <c r="C44" s="72" t="n">
         <v>64</v>
       </c>
-      <c r="D44" s="59">
+      <c r="D44" s="73">
         <f>IFERROR(C44-B44,"")</f>
         <v/>
       </c>
       <c r="E44" s="2" t="n"/>
     </row>
     <row r="45" ht="18" customHeight="1">
-      <c r="A45" s="54" t="inlineStr">
+      <c r="A45" s="68" t="inlineStr">
         <is>
           <t>Dec '25</t>
         </is>
       </c>
-      <c r="B45" s="38" t="n">
+      <c r="B45" s="52" t="n">
         <v>63.03</v>
       </c>
-      <c r="C45" s="55" t="n">
+      <c r="C45" s="69" t="n">
         <v>64</v>
       </c>
-      <c r="D45" s="56">
+      <c r="D45" s="70">
         <f>IFERROR(C45-B45,"")</f>
         <v/>
       </c>
-      <c r="E45" s="43" t="n"/>
+      <c r="E45" s="57" t="n"/>
     </row>
     <row r="46" ht="18" customHeight="1">
-      <c r="A46" s="57" t="inlineStr">
+      <c r="A46" s="71" t="inlineStr">
         <is>
           <t>Jan '26</t>
         </is>
       </c>
-      <c r="B46" s="45" t="n">
+      <c r="B46" s="59" t="n">
         <v>24.95</v>
       </c>
-      <c r="C46" s="58" t="n">
+      <c r="C46" s="72" t="n">
         <v>64</v>
       </c>
-      <c r="D46" s="59">
+      <c r="D46" s="73">
         <f>IFERROR(C46-B46,"")</f>
         <v/>
       </c>
       <c r="E46" s="2" t="n"/>
     </row>
     <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="54" t="inlineStr">
+      <c r="A47" s="68" t="inlineStr">
         <is>
           <t>Feb '26</t>
         </is>
       </c>
-      <c r="B47" s="38" t="n">
+      <c r="B47" s="52" t="n">
         <v>24.95</v>
       </c>
-      <c r="C47" s="55" t="n">
+      <c r="C47" s="69" t="n">
         <v>64</v>
       </c>
-      <c r="D47" s="56">
+      <c r="D47" s="70">
         <f>IFERROR(C47-B47,"")</f>
         <v/>
       </c>
-      <c r="E47" s="43" t="n"/>
+      <c r="E47" s="57" t="n"/>
     </row>
     <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="57" t="inlineStr">
+      <c r="A48" s="71" t="inlineStr">
         <is>
           <t>Mar '26</t>
         </is>
       </c>
-      <c r="B48" s="45" t="n">
+      <c r="B48" s="59" t="n">
         <v>24.95</v>
       </c>
-      <c r="C48" s="58" t="n">
+      <c r="C48" s="72" t="n">
         <v>64</v>
       </c>
-      <c r="D48" s="59">
+      <c r="D48" s="73">
         <f>IFERROR(C48-B48,"")</f>
         <v/>
       </c>
       <c r="E48" s="2" t="n"/>
     </row>
     <row r="49" ht="18" customHeight="1">
-      <c r="A49" s="54" t="inlineStr">
+      <c r="A49" s="68" t="inlineStr">
         <is>
           <t>Apr '26</t>
         </is>
       </c>
-      <c r="B49" s="38" t="n">
+      <c r="B49" s="52" t="n">
         <v>24.95</v>
       </c>
-      <c r="C49" s="55" t="n">
+      <c r="C49" s="69" t="n">
         <v>64</v>
       </c>
-      <c r="D49" s="56">
+      <c r="D49" s="70">
         <f>IFERROR(C49-B49,"")</f>
         <v/>
       </c>
-      <c r="E49" s="43" t="n"/>
+      <c r="E49" s="57" t="n"/>
     </row>
     <row r="50" ht="18" customHeight="1">
-      <c r="A50" s="57" t="inlineStr">
+      <c r="A50" s="71" t="inlineStr">
         <is>
           <t>Jun '26</t>
         </is>
       </c>
-      <c r="B50" s="45" t="n">
+      <c r="B50" s="59" t="n">
         <v>24.95</v>
       </c>
-      <c r="C50" s="58" t="n">
+      <c r="C50" s="72" t="n">
         <v>64</v>
       </c>
-      <c r="D50" s="59">
+      <c r="D50" s="73">
         <f>IFERROR(C50-B50,"")</f>
         <v/>
       </c>
       <c r="E50" s="2" t="n"/>
     </row>
     <row r="51" ht="22" customHeight="1">
-      <c r="A51" s="60" t="inlineStr">
+      <c r="A51" s="74" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B51" s="61">
+      <c r="B51" s="75">
         <f>SUM(B39:B50)</f>
         <v/>
       </c>
-      <c r="C51" s="61" t="n">
+      <c r="C51" s="75" t="n">
         <v>768</v>
       </c>
-      <c r="D51" s="62">
+      <c r="D51" s="76">
         <f>C51-B51</f>
         <v/>
       </c>
     </row>
     <row r="54" ht="26" customHeight="1">
-      <c r="A54" s="65" t="inlineStr">
+      <c r="A54" s="79" t="inlineStr">
         <is>
           <t>TRASH  ·  fund $23/mo  ·  avg $22  ·  cushion $1/mo</t>
         </is>
       </c>
     </row>
     <row r="55" ht="20" customHeight="1">
-      <c r="A55" s="44" t="inlineStr">
+      <c r="A55" s="58" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B55" s="44" t="inlineStr">
+      <c r="B55" s="58" t="inlineStr">
         <is>
           <t>Actual</t>
         </is>
       </c>
-      <c r="C55" s="44" t="inlineStr">
+      <c r="C55" s="58" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="D55" s="44" t="inlineStr">
+      <c r="D55" s="58" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="E55" s="44" t="inlineStr">
+      <c r="E55" s="58" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="56" ht="18" customHeight="1">
-      <c r="A56" s="54" t="inlineStr">
+      <c r="A56" s="68" t="inlineStr">
         <is>
           <t>Jun '25</t>
         </is>
       </c>
-      <c r="B56" s="38" t="n">
+      <c r="B56" s="52" t="n">
         <v>21.37</v>
       </c>
-      <c r="C56" s="55" t="n">
+      <c r="C56" s="69" t="n">
         <v>23</v>
       </c>
-      <c r="D56" s="56">
+      <c r="D56" s="70">
         <f>IFERROR(C56-B56,"")</f>
         <v/>
       </c>
-      <c r="E56" s="43" t="n"/>
+      <c r="E56" s="57" t="n"/>
     </row>
     <row r="57" ht="18" customHeight="1">
-      <c r="A57" s="57" t="inlineStr">
+      <c r="A57" s="71" t="inlineStr">
         <is>
           <t>Jul '25</t>
         </is>
       </c>
-      <c r="B57" s="45" t="n">
+      <c r="B57" s="59" t="n">
         <v>24.77</v>
       </c>
-      <c r="C57" s="58" t="n">
+      <c r="C57" s="72" t="n">
         <v>23</v>
       </c>
-      <c r="D57" s="59">
+      <c r="D57" s="73">
         <f>IFERROR(C57-B57,"")</f>
         <v/>
       </c>
       <c r="E57" s="2" t="n"/>
     </row>
     <row r="58" ht="18" customHeight="1">
-      <c r="A58" s="54" t="inlineStr">
+      <c r="A58" s="68" t="inlineStr">
         <is>
           <t>Aug '25</t>
         </is>
       </c>
-      <c r="B58" s="38" t="n"/>
-      <c r="C58" s="55" t="n">
+      <c r="B58" s="52" t="n"/>
+      <c r="C58" s="69" t="n">
         <v>23</v>
       </c>
-      <c r="D58" s="56">
+      <c r="D58" s="70">
         <f>IFERROR(C58-B58,"")</f>
         <v/>
       </c>
-      <c r="E58" s="43" t="n"/>
+      <c r="E58" s="57" t="n"/>
     </row>
     <row r="59" ht="18" customHeight="1">
-      <c r="A59" s="57" t="inlineStr">
+      <c r="A59" s="71" t="inlineStr">
         <is>
           <t>Sep '25</t>
         </is>
       </c>
-      <c r="B59" s="45" t="n">
+      <c r="B59" s="59" t="n">
         <v>21.37</v>
       </c>
-      <c r="C59" s="58" t="n">
+      <c r="C59" s="72" t="n">
         <v>23</v>
       </c>
-      <c r="D59" s="59">
+      <c r="D59" s="73">
         <f>IFERROR(C59-B59,"")</f>
         <v/>
       </c>
       <c r="E59" s="2" t="n"/>
     </row>
     <row r="60" ht="18" customHeight="1">
-      <c r="A60" s="54" t="inlineStr">
+      <c r="A60" s="68" t="inlineStr">
         <is>
           <t>Oct '25</t>
         </is>
       </c>
-      <c r="B60" s="38" t="n">
+      <c r="B60" s="52" t="n">
         <v>21.37</v>
       </c>
-      <c r="C60" s="55" t="n">
+      <c r="C60" s="69" t="n">
         <v>23</v>
       </c>
-      <c r="D60" s="56">
+      <c r="D60" s="70">
         <f>IFERROR(C60-B60,"")</f>
         <v/>
       </c>
-      <c r="E60" s="43" t="n"/>
+      <c r="E60" s="57" t="n"/>
     </row>
     <row r="61" ht="18" customHeight="1">
-      <c r="A61" s="57" t="inlineStr">
+      <c r="A61" s="71" t="inlineStr">
         <is>
           <t>Nov '25</t>
         </is>
       </c>
-      <c r="B61" s="45" t="n">
+      <c r="B61" s="59" t="n">
         <v>21.37</v>
       </c>
-      <c r="C61" s="58" t="n">
+      <c r="C61" s="72" t="n">
         <v>23</v>
       </c>
-      <c r="D61" s="59">
+      <c r="D61" s="73">
         <f>IFERROR(C61-B61,"")</f>
         <v/>
       </c>
       <c r="E61" s="2" t="n"/>
     </row>
     <row r="62" ht="18" customHeight="1">
-      <c r="A62" s="54" t="inlineStr">
+      <c r="A62" s="68" t="inlineStr">
         <is>
           <t>Dec '25</t>
         </is>
       </c>
-      <c r="B62" s="38" t="n">
+      <c r="B62" s="52" t="n">
         <v>21.37</v>
       </c>
-      <c r="C62" s="55" t="n">
+      <c r="C62" s="69" t="n">
         <v>23</v>
       </c>
-      <c r="D62" s="56">
+      <c r="D62" s="70">
         <f>IFERROR(C62-B62,"")</f>
         <v/>
       </c>
-      <c r="E62" s="43" t="n"/>
+      <c r="E62" s="57" t="n"/>
     </row>
     <row r="63" ht="18" customHeight="1">
-      <c r="A63" s="57" t="inlineStr">
+      <c r="A63" s="71" t="inlineStr">
         <is>
           <t>Jan '26</t>
         </is>
       </c>
-      <c r="B63" s="45" t="n">
+      <c r="B63" s="59" t="n">
         <v>22.01</v>
       </c>
-      <c r="C63" s="58" t="n">
+      <c r="C63" s="72" t="n">
         <v>23</v>
       </c>
-      <c r="D63" s="59">
+      <c r="D63" s="73">
         <f>IFERROR(C63-B63,"")</f>
         <v/>
       </c>
       <c r="E63" s="2" t="n"/>
     </row>
     <row r="64" ht="18" customHeight="1">
-      <c r="A64" s="54" t="inlineStr">
+      <c r="A64" s="68" t="inlineStr">
         <is>
           <t>Feb '26</t>
         </is>
       </c>
-      <c r="B64" s="38" t="n">
+      <c r="B64" s="52" t="n">
         <v>22.01</v>
       </c>
-      <c r="C64" s="55" t="n">
+      <c r="C64" s="69" t="n">
         <v>23</v>
       </c>
-      <c r="D64" s="56">
+      <c r="D64" s="70">
         <f>IFERROR(C64-B64,"")</f>
         <v/>
       </c>
-      <c r="E64" s="43" t="n"/>
+      <c r="E64" s="57" t="n"/>
     </row>
     <row r="65" ht="18" customHeight="1">
-      <c r="A65" s="57" t="inlineStr">
+      <c r="A65" s="71" t="inlineStr">
         <is>
           <t>Mar '26</t>
         </is>
       </c>
-      <c r="B65" s="45" t="n">
+      <c r="B65" s="59" t="n">
         <v>22.01</v>
       </c>
-      <c r="C65" s="58" t="n">
+      <c r="C65" s="72" t="n">
         <v>23</v>
       </c>
-      <c r="D65" s="59">
+      <c r="D65" s="73">
         <f>IFERROR(C65-B65,"")</f>
         <v/>
       </c>
       <c r="E65" s="2" t="n"/>
     </row>
     <row r="66" ht="18" customHeight="1">
-      <c r="A66" s="54" t="inlineStr">
+      <c r="A66" s="68" t="inlineStr">
         <is>
           <t>Apr '26</t>
         </is>
       </c>
-      <c r="B66" s="38" t="n">
+      <c r="B66" s="52" t="n">
         <v>22.01</v>
       </c>
-      <c r="C66" s="55" t="n">
+      <c r="C66" s="69" t="n">
         <v>23</v>
       </c>
-      <c r="D66" s="56">
+      <c r="D66" s="70">
         <f>IFERROR(C66-B66,"")</f>
         <v/>
       </c>
-      <c r="E66" s="43" t="n"/>
+      <c r="E66" s="57" t="n"/>
     </row>
     <row r="67" ht="18" customHeight="1">
-      <c r="A67" s="57" t="inlineStr">
+      <c r="A67" s="71" t="inlineStr">
         <is>
           <t>Jun '26</t>
         </is>
       </c>
-      <c r="B67" s="45" t="n">
+      <c r="B67" s="59" t="n">
         <v>22.01</v>
       </c>
-      <c r="C67" s="58" t="n">
+      <c r="C67" s="72" t="n">
         <v>23</v>
       </c>
-      <c r="D67" s="59">
+      <c r="D67" s="73">
         <f>IFERROR(C67-B67,"")</f>
         <v/>
       </c>
       <c r="E67" s="2" t="n"/>
     </row>
     <row r="68" ht="22" customHeight="1">
-      <c r="A68" s="60" t="inlineStr">
+      <c r="A68" s="74" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B68" s="61">
+      <c r="B68" s="75">
         <f>SUM(B56:B67)</f>
         <v/>
       </c>
-      <c r="C68" s="61" t="n">
+      <c r="C68" s="75" t="n">
         <v>276</v>
       </c>
-      <c r="D68" s="62">
+      <c r="D68" s="76">
         <f>C68-B68</f>
         <v/>
       </c>
@@ -3815,7 +4292,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="52" t="inlineStr">
+      <c r="A1" s="66" t="inlineStr">
         <is>
           <t>BILL CALENDAR — ALIGN TO PAYDAY</t>
         </is>
@@ -3829,54 +4306,54 @@
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="B4" s="28" t="inlineStr">
+      <c r="B4" s="42" t="inlineStr">
         <is>
           <t>BILL</t>
         </is>
       </c>
-      <c r="C4" s="28" t="inlineStr">
+      <c r="C4" s="42" t="inlineStr">
         <is>
           <t>AMOUNT</t>
         </is>
       </c>
-      <c r="D4" s="28" t="inlineStr">
+      <c r="D4" s="42" t="inlineStr">
         <is>
           <t>CURRENT DUE</t>
         </is>
       </c>
-      <c r="E4" s="28" t="inlineStr">
+      <c r="E4" s="42" t="inlineStr">
         <is>
           <t>TARGET DUE</t>
         </is>
       </c>
-      <c r="F4" s="28" t="inlineStr">
+      <c r="F4" s="42" t="inlineStr">
         <is>
           <t>NOTES</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="B5" s="66" t="inlineStr">
+      <c r="B5" s="80" t="inlineStr">
         <is>
           <t>FIXED BILLS — auto-pay from SoFi checking</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="B6" s="67" t="inlineStr">
+      <c r="B6" s="81" t="inlineStr">
         <is>
           <t>Mortgage</t>
         </is>
       </c>
-      <c r="C6" s="45" t="n">
+      <c r="C6" s="59" t="n">
         <v>837</v>
       </c>
-      <c r="D6" s="68" t="inlineStr">
+      <c r="D6" s="82" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E6" s="69" t="inlineStr">
+      <c r="E6" s="83" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3888,20 +4365,20 @@
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="B7" s="70" t="inlineStr">
+      <c r="B7" s="84" t="inlineStr">
         <is>
           <t>House insurance</t>
         </is>
       </c>
-      <c r="C7" s="38" t="n">
+      <c r="C7" s="52" t="n">
         <v>190</v>
       </c>
-      <c r="D7" s="71" t="inlineStr">
+      <c r="D7" s="85" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E7" s="72" t="inlineStr">
+      <c r="E7" s="86" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3913,20 +4390,20 @@
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="B8" s="67" t="inlineStr">
+      <c r="B8" s="81" t="inlineStr">
         <is>
           <t>Auto insurance</t>
         </is>
       </c>
-      <c r="C8" s="45" t="n">
+      <c r="C8" s="59" t="n">
         <v>79</v>
       </c>
-      <c r="D8" s="68" t="inlineStr">
+      <c r="D8" s="82" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E8" s="69" t="inlineStr">
+      <c r="E8" s="83" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3938,20 +4415,20 @@
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="B9" s="70" t="inlineStr">
+      <c r="B9" s="84" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="C9" s="38" t="n">
+      <c r="C9" s="52" t="n">
         <v>55</v>
       </c>
-      <c r="D9" s="71" t="inlineStr">
+      <c r="D9" s="85" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E9" s="72" t="inlineStr">
+      <c r="E9" s="86" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3963,20 +4440,20 @@
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="B10" s="67" t="inlineStr">
+      <c r="B10" s="81" t="inlineStr">
         <is>
           <t>Property tax set-aside</t>
         </is>
       </c>
-      <c r="C10" s="45" t="n">
+      <c r="C10" s="59" t="n">
         <v>54</v>
       </c>
-      <c r="D10" s="68" t="inlineStr">
+      <c r="D10" s="82" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E10" s="69" t="inlineStr">
+      <c r="E10" s="83" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3988,27 +4465,27 @@
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="B12" s="73" t="inlineStr">
+      <c r="B12" s="87" t="inlineStr">
         <is>
           <t>FLEX UTILITIES — auto-draft from Flex account</t>
         </is>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="B13" s="67" t="inlineStr">
+      <c r="B13" s="81" t="inlineStr">
         <is>
           <t>Power</t>
         </is>
       </c>
-      <c r="C13" s="45" t="n">
+      <c r="C13" s="59" t="n">
         <v>453</v>
       </c>
-      <c r="D13" s="68" t="inlineStr">
+      <c r="D13" s="82" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E13" s="69" t="inlineStr">
+      <c r="E13" s="83" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -4020,20 +4497,20 @@
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="B14" s="70" t="inlineStr">
+      <c r="B14" s="84" t="inlineStr">
         <is>
           <t>Water</t>
         </is>
       </c>
-      <c r="C14" s="38" t="n">
+      <c r="C14" s="52" t="n">
         <v>90</v>
       </c>
-      <c r="D14" s="71" t="inlineStr">
+      <c r="D14" s="85" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E14" s="72" t="inlineStr">
+      <c r="E14" s="86" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -4045,20 +4522,20 @@
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="B15" s="67" t="inlineStr">
+      <c r="B15" s="81" t="inlineStr">
         <is>
           <t>Internet</t>
         </is>
       </c>
-      <c r="C15" s="45" t="n">
+      <c r="C15" s="59" t="n">
         <v>64</v>
       </c>
-      <c r="D15" s="68" t="inlineStr">
+      <c r="D15" s="82" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E15" s="69" t="inlineStr">
+      <c r="E15" s="83" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -4070,20 +4547,20 @@
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="B16" s="70" t="inlineStr">
+      <c r="B16" s="84" t="inlineStr">
         <is>
           <t>Trash</t>
         </is>
       </c>
-      <c r="C16" s="38" t="n">
+      <c r="C16" s="52" t="n">
         <v>23</v>
       </c>
-      <c r="D16" s="71" t="inlineStr">
+      <c r="D16" s="85" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E16" s="72" t="inlineStr">
+      <c r="E16" s="86" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -4102,7 +4579,7 @@
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
-      <c r="B20" s="74" t="inlineStr">
+      <c r="B20" s="88" t="inlineStr">
         <is>
           <t>● Move the due dates</t>
         </is>
@@ -4116,7 +4593,7 @@
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
-      <c r="B22" s="75" t="inlineStr">
+      <c r="B22" s="89" t="inlineStr">
         <is>
           <t>● Keep buffers</t>
         </is>
@@ -4130,7 +4607,7 @@
       </c>
     </row>
     <row r="24" ht="15" customHeight="1">
-      <c r="B24" s="74" t="inlineStr">
+      <c r="B24" s="88" t="inlineStr">
         <is>
           <t>● Group by paycheck</t>
         </is>

</xml_diff>

<commit_message>
Fix $0.00 display: pre-compute all static budget values in Python
openpyxl stores formulas without cached values, so any viewer that
doesn't auto-recalculate (previews, some mobile apps) showed $0.00.

Fix: replace every formula that referenced only hard-coded inputs with
Python-computed values stored directly in the cells. This covers all
summaries (income, fixed, flex, leftover, SE reserve, sinking, income
trajectory, revised bottom line). Savings-goals cells (EF/Septic
progress) retain formulas since they reference the user-editable
savings balance input and will recompute correctly when that cell is
changed in any spreadsheet app.

Also adds wb.calculation.fullCalcOnLoad = True for Excel compatibility.
</commit_message>
<xml_diff>
--- a/utilities/Budget_System.xlsx
+++ b/utilities/Budget_System.xlsx
@@ -1124,9 +1124,8 @@
           <t>TOTAL SPENDABLE</t>
         </is>
       </c>
-      <c r="C8" s="8">
-        <f>C5+C6+C7</f>
-        <v/>
+      <c r="C8" s="8" t="n">
+        <v>3668</v>
       </c>
       <c r="D8" s="9" t="n"/>
     </row>
@@ -1212,9 +1211,8 @@
           <t>FIXED TOTAL</t>
         </is>
       </c>
-      <c r="C17" s="8">
-        <f>SUM(C12:C16)</f>
-        <v/>
+      <c r="C17" s="8" t="n">
+        <v>1215</v>
       </c>
       <c r="D17" s="9" t="n"/>
     </row>
@@ -1288,9 +1286,8 @@
           <t>UTILITIES SUBTOTAL  (fund flat)</t>
         </is>
       </c>
-      <c r="C24" s="8">
-        <f>SUM(C20:C23)</f>
-        <v/>
+      <c r="C24" s="8" t="n">
+        <v>630</v>
       </c>
       <c r="D24" s="9" t="n"/>
     </row>
@@ -1326,9 +1323,8 @@
           <t>FLEX TOTAL</t>
         </is>
       </c>
-      <c r="C27" s="8">
-        <f>C24+430+400</f>
-        <v/>
+      <c r="C27" s="8" t="n">
+        <v>1460</v>
       </c>
       <c r="D27" s="9" t="n"/>
     </row>
@@ -1361,9 +1357,8 @@
           <t>Leftover after fixed + flex</t>
         </is>
       </c>
-      <c r="C31" s="8">
-        <f>C8-C17-C27</f>
-        <v/>
+      <c r="C31" s="8" t="n">
+        <v>993</v>
       </c>
       <c r="D31" s="9" t="n"/>
     </row>
@@ -1373,9 +1368,8 @@
           <t>⚠  If Shane's $628 stops → leftover</t>
         </is>
       </c>
-      <c r="C32" s="19">
-        <f>C31-628</f>
-        <v/>
+      <c r="C32" s="19" t="n">
+        <v>365</v>
       </c>
       <c r="D32" s="20" t="inlineStr">
         <is>
@@ -1412,9 +1406,8 @@
           <t>SAVINGS — SoFi Vaults  (what's left)</t>
         </is>
       </c>
-      <c r="C36" s="22">
-        <f>C31-C35</f>
-        <v/>
+      <c r="C36" s="22" t="n">
+        <v>493</v>
       </c>
       <c r="D36" s="23" t="inlineStr">
         <is>
@@ -1466,9 +1459,8 @@
           <t>Hidden savings in flex (approx.)</t>
         </is>
       </c>
-      <c r="C41" s="25">
-        <f>C39+C40</f>
-        <v/>
+      <c r="C41" s="25" t="n">
+        <v>84</v>
       </c>
       <c r="D41" s="26" t="n"/>
     </row>
@@ -1486,9 +1478,8 @@
           <t>Side work gross  (from income above)</t>
         </is>
       </c>
-      <c r="C44" s="13">
-        <f>C6</f>
-        <v/>
+      <c r="C44" s="13" t="n">
+        <v>480</v>
       </c>
       <c r="D44" s="16" t="inlineStr">
         <is>
@@ -1502,9 +1493,8 @@
           <t>Monthly reserve  (28% — SE tax 15.3% + income tax est.)</t>
         </is>
       </c>
-      <c r="C45" s="29">
-        <f>C44*0.28</f>
-        <v/>
+      <c r="C45" s="29" t="n">
+        <v>134.4</v>
       </c>
       <c r="D45" s="30" t="inlineStr">
         <is>
@@ -1518,9 +1508,8 @@
           <t>True spendable from side work</t>
         </is>
       </c>
-      <c r="C46" s="13">
-        <f>C44-C45</f>
-        <v/>
+      <c r="C46" s="13" t="n">
+        <v>345.6</v>
       </c>
       <c r="D46" s="16" t="inlineStr">
         <is>
@@ -1587,9 +1576,8 @@
           <t>SINKING TOTAL  — set aside monthly</t>
         </is>
       </c>
-      <c r="C52" s="8">
-        <f>SUM(C49:C51)</f>
-        <v/>
+      <c r="C52" s="8" t="n">
+        <v>92</v>
       </c>
       <c r="D52" s="31" t="inlineStr">
         <is>
@@ -1656,9 +1644,8 @@
           <t>Est. take-home at $22/hr  (40hr/wk, ~72% net)</t>
         </is>
       </c>
-      <c r="C58" s="5">
-        <f>22*40*52/12*0.72</f>
-        <v/>
+      <c r="C58" s="5" t="n">
+        <v>2745.6</v>
       </c>
       <c r="D58" s="6" t="inlineStr">
         <is>
@@ -1672,9 +1659,8 @@
           <t>Monthly income gain at target</t>
         </is>
       </c>
-      <c r="C59" s="25">
-        <f>C58-C56</f>
-        <v/>
+      <c r="C59" s="25" t="n">
+        <v>185.6</v>
       </c>
       <c r="D59" s="23" t="inlineStr">
         <is>
@@ -1815,9 +1801,8 @@
           <t>Gross leftover  (after fixed + flex)</t>
         </is>
       </c>
-      <c r="C75" s="13">
-        <f>C31</f>
-        <v/>
+      <c r="C75" s="13" t="n">
+        <v>993</v>
       </c>
       <c r="D75" s="14" t="n"/>
     </row>
@@ -1827,9 +1812,8 @@
           <t xml:space="preserve">  Less: SE tax reserve</t>
         </is>
       </c>
-      <c r="C76" s="5">
-        <f>-C45</f>
-        <v/>
+      <c r="C76" s="5" t="n">
+        <v>-134.4</v>
       </c>
       <c r="D76" s="10" t="n"/>
     </row>
@@ -1839,9 +1823,8 @@
           <t xml:space="preserve">  Less: sinking funds</t>
         </is>
       </c>
-      <c r="C77" s="13">
-        <f>-C52</f>
-        <v/>
+      <c r="C77" s="13" t="n">
+        <v>-92</v>
       </c>
       <c r="D77" s="14" t="n"/>
     </row>
@@ -1851,9 +1834,8 @@
           <t>TRUE MONTHLY AVAILABLE</t>
         </is>
       </c>
-      <c r="C78" s="8">
-        <f>C31-C45-C52</f>
-        <v/>
+      <c r="C78" s="8" t="n">
+        <v>766.6</v>
       </c>
       <c r="D78" s="9" t="n"/>
     </row>
@@ -1863,9 +1845,8 @@
           <t xml:space="preserve">  If Shane's $628 stops → true available</t>
         </is>
       </c>
-      <c r="C79" s="19">
-        <f>C78-628</f>
-        <v/>
+      <c r="C79" s="19" t="n">
+        <v>138.6</v>
       </c>
       <c r="D79" s="20" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix Monthly Check-In: pre-compute all historical values, fix sweep formula
Three issues fixed:
1. All formula cells (Total Actual, Net, Buffer Bal, Sweep, Totals,
   Averages) showed $0.00 — replaced with Python-computed values for
   all 12 historical months so any viewer displays correct numbers.
2. Sweep formula bug: prev_buf_row was updated before the sweep check,
   making it always use the first-row variant (sweep = all surplus with
   no refill deduction). Fixed by computing both I and J before updating
   prev_buf_row, and referencing the previous row's buffer for refill math.
3. Future-row formula changed from IFERROR(SUM) to IF(COUNTA=0,"",SUM)
   so blank future months show empty instead of $0.00 Total Actual.
Totals and Averages rows also pre-computed; G and J columns added to averages.
</commit_message>
<xml_diff>
--- a/utilities/Budget_System.xlsx
+++ b/utilities/Budget_System.xlsx
@@ -1986,24 +1986,20 @@
       <c r="E5" s="52" t="n">
         <v>21.37</v>
       </c>
-      <c r="F5" s="53">
-        <f>IFERROR(SUM(B5:E5),"")</f>
-        <v/>
+      <c r="F5" s="53" t="n">
+        <v>455.46</v>
       </c>
       <c r="G5" s="54" t="n">
         <v>630</v>
       </c>
-      <c r="H5" s="55">
-        <f>IFERROR(G5-F5,"")</f>
-        <v/>
-      </c>
-      <c r="I5" s="52">
-        <f>IFERROR(MAX(0,MIN(167.63,167.63+H5)),"")</f>
-        <v/>
-      </c>
-      <c r="J5" s="56">
-        <f>IFERROR(MAX(0,H5-MAX(0,167.63-167.63)),"")</f>
-        <v/>
+      <c r="H5" s="55" t="n">
+        <v>174.54</v>
+      </c>
+      <c r="I5" s="52" t="n">
+        <v>167.63</v>
+      </c>
+      <c r="J5" s="56" t="n">
+        <v>174.54</v>
       </c>
       <c r="K5" s="57" t="n"/>
     </row>
@@ -2025,24 +2021,20 @@
       <c r="E6" s="59" t="n">
         <v>24.77</v>
       </c>
-      <c r="F6" s="60">
-        <f>IFERROR(SUM(B6:E6),"")</f>
-        <v/>
+      <c r="F6" s="60" t="n">
+        <v>536.24</v>
       </c>
       <c r="G6" s="61" t="n">
         <v>630</v>
       </c>
-      <c r="H6" s="62">
-        <f>IFERROR(G6-F6,"")</f>
-        <v/>
-      </c>
-      <c r="I6" s="59">
-        <f>IFERROR(MAX(0,MIN(167.63,I5+H6)),"")</f>
-        <v/>
-      </c>
-      <c r="J6" s="63">
-        <f>IFERROR(MAX(0,H6-MAX(0,167.63-167.63)),"")</f>
-        <v/>
+      <c r="H6" s="62" t="n">
+        <v>93.76000000000001</v>
+      </c>
+      <c r="I6" s="59" t="n">
+        <v>167.63</v>
+      </c>
+      <c r="J6" s="63" t="n">
+        <v>93.76000000000001</v>
       </c>
       <c r="K6" s="2" t="n"/>
     </row>
@@ -2062,24 +2054,20 @@
         <v>42.98</v>
       </c>
       <c r="E7" s="52" t="n"/>
-      <c r="F7" s="53">
-        <f>IFERROR(SUM(B7:E7),"")</f>
-        <v/>
+      <c r="F7" s="53" t="n">
+        <v>496.6</v>
       </c>
       <c r="G7" s="54" t="n">
         <v>630</v>
       </c>
-      <c r="H7" s="55">
-        <f>IFERROR(G7-F7,"")</f>
-        <v/>
-      </c>
-      <c r="I7" s="52">
-        <f>IFERROR(MAX(0,MIN(167.63,I6+H7)),"")</f>
-        <v/>
-      </c>
-      <c r="J7" s="56">
-        <f>IFERROR(MAX(0,H7-MAX(0,167.63-167.63)),"")</f>
-        <v/>
+      <c r="H7" s="55" t="n">
+        <v>133.4</v>
+      </c>
+      <c r="I7" s="52" t="n">
+        <v>167.63</v>
+      </c>
+      <c r="J7" s="56" t="n">
+        <v>133.4</v>
       </c>
       <c r="K7" s="57" t="n"/>
     </row>
@@ -2101,24 +2089,20 @@
       <c r="E8" s="59" t="n">
         <v>21.37</v>
       </c>
-      <c r="F8" s="60">
-        <f>IFERROR(SUM(B8:E8),"")</f>
-        <v/>
+      <c r="F8" s="60" t="n">
+        <v>499.51</v>
       </c>
       <c r="G8" s="61" t="n">
         <v>630</v>
       </c>
-      <c r="H8" s="62">
-        <f>IFERROR(G8-F8,"")</f>
-        <v/>
-      </c>
-      <c r="I8" s="59">
-        <f>IFERROR(MAX(0,MIN(167.63,I7+H8)),"")</f>
-        <v/>
-      </c>
-      <c r="J8" s="63">
-        <f>IFERROR(MAX(0,H8-MAX(0,167.63-167.63)),"")</f>
-        <v/>
+      <c r="H8" s="62" t="n">
+        <v>130.49</v>
+      </c>
+      <c r="I8" s="59" t="n">
+        <v>167.63</v>
+      </c>
+      <c r="J8" s="63" t="n">
+        <v>130.49</v>
       </c>
       <c r="K8" s="2" t="n"/>
     </row>
@@ -2140,24 +2124,20 @@
       <c r="E9" s="52" t="n">
         <v>21.37</v>
       </c>
-      <c r="F9" s="53">
-        <f>IFERROR(SUM(B9:E9),"")</f>
-        <v/>
+      <c r="F9" s="53" t="n">
+        <v>368.72</v>
       </c>
       <c r="G9" s="54" t="n">
         <v>630</v>
       </c>
-      <c r="H9" s="55">
-        <f>IFERROR(G9-F9,"")</f>
-        <v/>
-      </c>
-      <c r="I9" s="52">
-        <f>IFERROR(MAX(0,MIN(167.63,I8+H9)),"")</f>
-        <v/>
-      </c>
-      <c r="J9" s="56">
-        <f>IFERROR(MAX(0,H9-MAX(0,167.63-167.63)),"")</f>
-        <v/>
+      <c r="H9" s="55" t="n">
+        <v>261.28</v>
+      </c>
+      <c r="I9" s="52" t="n">
+        <v>167.63</v>
+      </c>
+      <c r="J9" s="56" t="n">
+        <v>261.28</v>
       </c>
       <c r="K9" s="57" t="n"/>
     </row>
@@ -2179,24 +2159,20 @@
       <c r="E10" s="59" t="n">
         <v>21.37</v>
       </c>
-      <c r="F10" s="60">
-        <f>IFERROR(SUM(B10:E10),"")</f>
-        <v/>
+      <c r="F10" s="60" t="n">
+        <v>384.87</v>
       </c>
       <c r="G10" s="61" t="n">
         <v>630</v>
       </c>
-      <c r="H10" s="62">
-        <f>IFERROR(G10-F10,"")</f>
-        <v/>
-      </c>
-      <c r="I10" s="59">
-        <f>IFERROR(MAX(0,MIN(167.63,I9+H10)),"")</f>
-        <v/>
-      </c>
-      <c r="J10" s="63">
-        <f>IFERROR(MAX(0,H10-MAX(0,167.63-167.63)),"")</f>
-        <v/>
+      <c r="H10" s="62" t="n">
+        <v>245.13</v>
+      </c>
+      <c r="I10" s="59" t="n">
+        <v>167.63</v>
+      </c>
+      <c r="J10" s="63" t="n">
+        <v>245.13</v>
       </c>
       <c r="K10" s="2" t="n"/>
     </row>
@@ -2218,24 +2194,20 @@
       <c r="E11" s="52" t="n">
         <v>21.37</v>
       </c>
-      <c r="F11" s="53">
-        <f>IFERROR(SUM(B11:E11),"")</f>
-        <v/>
+      <c r="F11" s="53" t="n">
+        <v>543.5700000000001</v>
       </c>
       <c r="G11" s="54" t="n">
         <v>630</v>
       </c>
-      <c r="H11" s="55">
-        <f>IFERROR(G11-F11,"")</f>
-        <v/>
-      </c>
-      <c r="I11" s="52">
-        <f>IFERROR(MAX(0,MIN(167.63,I10+H11)),"")</f>
-        <v/>
-      </c>
-      <c r="J11" s="56">
-        <f>IFERROR(MAX(0,H11-MAX(0,167.63-167.63)),"")</f>
-        <v/>
+      <c r="H11" s="55" t="n">
+        <v>86.43000000000001</v>
+      </c>
+      <c r="I11" s="52" t="n">
+        <v>167.63</v>
+      </c>
+      <c r="J11" s="56" t="n">
+        <v>86.43000000000001</v>
       </c>
       <c r="K11" s="57" t="n"/>
     </row>
@@ -2257,24 +2229,20 @@
       <c r="E12" s="59" t="n">
         <v>22.01</v>
       </c>
-      <c r="F12" s="60">
-        <f>IFERROR(SUM(B12:E12),"")</f>
-        <v/>
+      <c r="F12" s="60" t="n">
+        <v>629.38</v>
       </c>
       <c r="G12" s="61" t="n">
         <v>630</v>
       </c>
-      <c r="H12" s="62">
-        <f>IFERROR(G12-F12,"")</f>
-        <v/>
-      </c>
-      <c r="I12" s="59">
-        <f>IFERROR(MAX(0,MIN(167.63,I11+H12)),"")</f>
-        <v/>
-      </c>
-      <c r="J12" s="63">
-        <f>IFERROR(MAX(0,H12-MAX(0,167.63-167.63)),"")</f>
-        <v/>
+      <c r="H12" s="62" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="I12" s="59" t="n">
+        <v>167.63</v>
+      </c>
+      <c r="J12" s="63" t="n">
+        <v>0.62</v>
       </c>
       <c r="K12" s="2" t="n"/>
     </row>
@@ -2296,24 +2264,20 @@
       <c r="E13" s="52" t="n">
         <v>22.01</v>
       </c>
-      <c r="F13" s="53">
-        <f>IFERROR(SUM(B13:E13),"")</f>
-        <v/>
+      <c r="F13" s="53" t="n">
+        <v>466.21</v>
       </c>
       <c r="G13" s="54" t="n">
         <v>630</v>
       </c>
-      <c r="H13" s="55">
-        <f>IFERROR(G13-F13,"")</f>
-        <v/>
-      </c>
-      <c r="I13" s="52">
-        <f>IFERROR(MAX(0,MIN(167.63,I12+H13)),"")</f>
-        <v/>
-      </c>
-      <c r="J13" s="56">
-        <f>IFERROR(MAX(0,H13-MAX(0,167.63-167.63)),"")</f>
-        <v/>
+      <c r="H13" s="55" t="n">
+        <v>163.79</v>
+      </c>
+      <c r="I13" s="52" t="n">
+        <v>167.63</v>
+      </c>
+      <c r="J13" s="56" t="n">
+        <v>163.79</v>
       </c>
       <c r="K13" s="57" t="n"/>
     </row>
@@ -2335,24 +2299,20 @@
       <c r="E14" s="59" t="n">
         <v>22.01</v>
       </c>
-      <c r="F14" s="60">
-        <f>IFERROR(SUM(B14:E14),"")</f>
-        <v/>
+      <c r="F14" s="60" t="n">
+        <v>313.28</v>
       </c>
       <c r="G14" s="61" t="n">
         <v>630</v>
       </c>
-      <c r="H14" s="62">
-        <f>IFERROR(G14-F14,"")</f>
-        <v/>
-      </c>
-      <c r="I14" s="59">
-        <f>IFERROR(MAX(0,MIN(167.63,I13+H14)),"")</f>
-        <v/>
-      </c>
-      <c r="J14" s="63">
-        <f>IFERROR(MAX(0,H14-MAX(0,167.63-167.63)),"")</f>
-        <v/>
+      <c r="H14" s="62" t="n">
+        <v>316.72</v>
+      </c>
+      <c r="I14" s="59" t="n">
+        <v>167.63</v>
+      </c>
+      <c r="J14" s="63" t="n">
+        <v>316.72</v>
       </c>
       <c r="K14" s="2" t="n"/>
     </row>
@@ -2374,24 +2334,20 @@
       <c r="E15" s="52" t="n">
         <v>22.01</v>
       </c>
-      <c r="F15" s="53">
-        <f>IFERROR(SUM(B15:E15),"")</f>
-        <v/>
+      <c r="F15" s="53" t="n">
+        <v>339.47</v>
       </c>
       <c r="G15" s="54" t="n">
         <v>630</v>
       </c>
-      <c r="H15" s="55">
-        <f>IFERROR(G15-F15,"")</f>
-        <v/>
-      </c>
-      <c r="I15" s="52">
-        <f>IFERROR(MAX(0,MIN(167.63,I14+H15)),"")</f>
-        <v/>
-      </c>
-      <c r="J15" s="56">
-        <f>IFERROR(MAX(0,H15-MAX(0,167.63-167.63)),"")</f>
-        <v/>
+      <c r="H15" s="55" t="n">
+        <v>290.53</v>
+      </c>
+      <c r="I15" s="52" t="n">
+        <v>167.63</v>
+      </c>
+      <c r="J15" s="56" t="n">
+        <v>290.53</v>
       </c>
       <c r="K15" s="57" t="n"/>
     </row>
@@ -2406,24 +2362,20 @@
       <c r="D16" s="59" t="n"/>
       <c r="E16" s="59" t="n"/>
       <c r="F16" s="60">
-        <f>IFERROR(SUM(B16:E16),"")</f>
+        <f>IF(COUNTA(B16:E16)=0,"",SUM(B16:E16))</f>
         <v/>
       </c>
       <c r="G16" s="61" t="n">
         <v>630</v>
       </c>
       <c r="H16" s="62">
-        <f>IFERROR(G16-F16,"")</f>
-        <v/>
-      </c>
-      <c r="I16" s="59">
-        <f>IFERROR(MAX(0,MIN(167.63,I15+H16)),"")</f>
-        <v/>
-      </c>
-      <c r="J16" s="63">
-        <f>IFERROR(MAX(0,H16-MAX(0,167.63-167.63)),"")</f>
-        <v/>
-      </c>
+        <f>IF(F16="","",G16-F16)</f>
+        <v/>
+      </c>
+      <c r="I16" s="59" t="n">
+        <v>167.63</v>
+      </c>
+      <c r="J16" s="63" t="n"/>
       <c r="K16" s="2" t="n"/>
     </row>
     <row r="17" ht="20" customHeight="1">
@@ -2444,24 +2396,20 @@
       <c r="E17" s="52" t="n">
         <v>22.01</v>
       </c>
-      <c r="F17" s="53">
-        <f>IFERROR(SUM(B17:E17),"")</f>
-        <v/>
+      <c r="F17" s="53" t="n">
+        <v>434.51</v>
       </c>
       <c r="G17" s="54" t="n">
         <v>630</v>
       </c>
-      <c r="H17" s="55">
-        <f>IFERROR(G17-F17,"")</f>
-        <v/>
-      </c>
-      <c r="I17" s="52">
-        <f>IFERROR(MAX(0,MIN(167.63,I16+H17)),"")</f>
-        <v/>
-      </c>
-      <c r="J17" s="56">
-        <f>IFERROR(MAX(0,H17-MAX(0,167.63-167.63)),"")</f>
-        <v/>
+      <c r="H17" s="55" t="n">
+        <v>195.49</v>
+      </c>
+      <c r="I17" s="52" t="n">
+        <v>167.63</v>
+      </c>
+      <c r="J17" s="56" t="n">
+        <v>195.49</v>
       </c>
       <c r="K17" s="57" t="n"/>
     </row>
@@ -2476,22 +2424,22 @@
       <c r="D18" s="59" t="n"/>
       <c r="E18" s="59" t="n"/>
       <c r="F18" s="60">
-        <f>IFERROR(SUM(B18:E18),"")</f>
+        <f>IF(COUNTA(B18:E18)=0,"",SUM(B18:E18))</f>
         <v/>
       </c>
       <c r="G18" s="61" t="n">
         <v>630</v>
       </c>
       <c r="H18" s="62">
-        <f>IFERROR(G18-F18,"")</f>
+        <f>IF(F18="","",G18-F18)</f>
         <v/>
       </c>
       <c r="I18" s="59">
-        <f>IFERROR(MAX(0,MIN(167.63,I17+H18)),"")</f>
+        <f>IF(H18="","",MAX(0,MIN(167.63,I17+H18)))</f>
         <v/>
       </c>
       <c r="J18" s="63">
-        <f>IFERROR(MAX(0,H18-MAX(0,167.63-167.63)),"")</f>
+        <f>IF(H18="","",MAX(0,H18-MAX(0,167.63-I17)))</f>
         <v/>
       </c>
       <c r="K18" s="2" t="n"/>
@@ -2507,22 +2455,22 @@
       <c r="D19" s="52" t="n"/>
       <c r="E19" s="52" t="n"/>
       <c r="F19" s="53">
-        <f>IFERROR(SUM(B19:E19),"")</f>
+        <f>IF(COUNTA(B19:E19)=0,"",SUM(B19:E19))</f>
         <v/>
       </c>
       <c r="G19" s="54" t="n">
         <v>630</v>
       </c>
       <c r="H19" s="55">
-        <f>IFERROR(G19-F19,"")</f>
+        <f>IF(F19="","",G19-F19)</f>
         <v/>
       </c>
       <c r="I19" s="52">
-        <f>IFERROR(MAX(0,MIN(167.63,I18+H19)),"")</f>
+        <f>IF(H19="","",MAX(0,MIN(167.63,I18+H19)))</f>
         <v/>
       </c>
       <c r="J19" s="56">
-        <f>IFERROR(MAX(0,H19-MAX(0,167.63-167.63)),"")</f>
+        <f>IF(H19="","",MAX(0,H19-MAX(0,167.63-I18)))</f>
         <v/>
       </c>
       <c r="K19" s="57" t="n"/>
@@ -2538,22 +2486,22 @@
       <c r="D20" s="59" t="n"/>
       <c r="E20" s="59" t="n"/>
       <c r="F20" s="60">
-        <f>IFERROR(SUM(B20:E20),"")</f>
+        <f>IF(COUNTA(B20:E20)=0,"",SUM(B20:E20))</f>
         <v/>
       </c>
       <c r="G20" s="61" t="n">
         <v>630</v>
       </c>
       <c r="H20" s="62">
-        <f>IFERROR(G20-F20,"")</f>
+        <f>IF(F20="","",G20-F20)</f>
         <v/>
       </c>
       <c r="I20" s="59">
-        <f>IFERROR(MAX(0,MIN(167.63,I19+H20)),"")</f>
+        <f>IF(H20="","",MAX(0,MIN(167.63,I19+H20)))</f>
         <v/>
       </c>
       <c r="J20" s="63">
-        <f>IFERROR(MAX(0,H20-MAX(0,167.63-167.63)),"")</f>
+        <f>IF(H20="","",MAX(0,H20-MAX(0,167.63-I19)))</f>
         <v/>
       </c>
       <c r="K20" s="2" t="n"/>
@@ -2569,22 +2517,22 @@
       <c r="D21" s="52" t="n"/>
       <c r="E21" s="52" t="n"/>
       <c r="F21" s="53">
-        <f>IFERROR(SUM(B21:E21),"")</f>
+        <f>IF(COUNTA(B21:E21)=0,"",SUM(B21:E21))</f>
         <v/>
       </c>
       <c r="G21" s="54" t="n">
         <v>630</v>
       </c>
       <c r="H21" s="55">
-        <f>IFERROR(G21-F21,"")</f>
+        <f>IF(F21="","",G21-F21)</f>
         <v/>
       </c>
       <c r="I21" s="52">
-        <f>IFERROR(MAX(0,MIN(167.63,I20+H21)),"")</f>
+        <f>IF(H21="","",MAX(0,MIN(167.63,I20+H21)))</f>
         <v/>
       </c>
       <c r="J21" s="56">
-        <f>IFERROR(MAX(0,H21-MAX(0,167.63-167.63)),"")</f>
+        <f>IF(H21="","",MAX(0,H21-MAX(0,167.63-I20)))</f>
         <v/>
       </c>
       <c r="K21" s="57" t="n"/>
@@ -2600,22 +2548,22 @@
       <c r="D22" s="59" t="n"/>
       <c r="E22" s="59" t="n"/>
       <c r="F22" s="60">
-        <f>IFERROR(SUM(B22:E22),"")</f>
+        <f>IF(COUNTA(B22:E22)=0,"",SUM(B22:E22))</f>
         <v/>
       </c>
       <c r="G22" s="61" t="n">
         <v>630</v>
       </c>
       <c r="H22" s="62">
-        <f>IFERROR(G22-F22,"")</f>
+        <f>IF(F22="","",G22-F22)</f>
         <v/>
       </c>
       <c r="I22" s="59">
-        <f>IFERROR(MAX(0,MIN(167.63,I21+H22)),"")</f>
+        <f>IF(H22="","",MAX(0,MIN(167.63,I21+H22)))</f>
         <v/>
       </c>
       <c r="J22" s="63">
-        <f>IFERROR(MAX(0,H22-MAX(0,167.63-167.63)),"")</f>
+        <f>IF(H22="","",MAX(0,H22-MAX(0,167.63-I21)))</f>
         <v/>
       </c>
       <c r="K22" s="2" t="n"/>
@@ -2631,22 +2579,22 @@
       <c r="D23" s="52" t="n"/>
       <c r="E23" s="52" t="n"/>
       <c r="F23" s="53">
-        <f>IFERROR(SUM(B23:E23),"")</f>
+        <f>IF(COUNTA(B23:E23)=0,"",SUM(B23:E23))</f>
         <v/>
       </c>
       <c r="G23" s="54" t="n">
         <v>630</v>
       </c>
       <c r="H23" s="55">
-        <f>IFERROR(G23-F23,"")</f>
+        <f>IF(F23="","",G23-F23)</f>
         <v/>
       </c>
       <c r="I23" s="52">
-        <f>IFERROR(MAX(0,MIN(167.63,I22+H23)),"")</f>
+        <f>IF(H23="","",MAX(0,MIN(167.63,I22+H23)))</f>
         <v/>
       </c>
       <c r="J23" s="56">
-        <f>IFERROR(MAX(0,H23-MAX(0,167.63-167.63)),"")</f>
+        <f>IF(H23="","",MAX(0,H23-MAX(0,167.63-I22)))</f>
         <v/>
       </c>
       <c r="K23" s="57" t="n"/>
@@ -2662,22 +2610,22 @@
       <c r="D24" s="59" t="n"/>
       <c r="E24" s="59" t="n"/>
       <c r="F24" s="60">
-        <f>IFERROR(SUM(B24:E24),"")</f>
+        <f>IF(COUNTA(B24:E24)=0,"",SUM(B24:E24))</f>
         <v/>
       </c>
       <c r="G24" s="61" t="n">
         <v>630</v>
       </c>
       <c r="H24" s="62">
-        <f>IFERROR(G24-F24,"")</f>
+        <f>IF(F24="","",G24-F24)</f>
         <v/>
       </c>
       <c r="I24" s="59">
-        <f>IFERROR(MAX(0,MIN(167.63,I23+H24)),"")</f>
+        <f>IF(H24="","",MAX(0,MIN(167.63,I23+H24)))</f>
         <v/>
       </c>
       <c r="J24" s="63">
-        <f>IFERROR(MAX(0,H24-MAX(0,167.63-167.63)),"")</f>
+        <f>IF(H24="","",MAX(0,H24-MAX(0,167.63-I23)))</f>
         <v/>
       </c>
       <c r="K24" s="2" t="n"/>
@@ -2693,22 +2641,22 @@
       <c r="D25" s="52" t="n"/>
       <c r="E25" s="52" t="n"/>
       <c r="F25" s="53">
-        <f>IFERROR(SUM(B25:E25),"")</f>
+        <f>IF(COUNTA(B25:E25)=0,"",SUM(B25:E25))</f>
         <v/>
       </c>
       <c r="G25" s="54" t="n">
         <v>630</v>
       </c>
       <c r="H25" s="55">
-        <f>IFERROR(G25-F25,"")</f>
+        <f>IF(F25="","",G25-F25)</f>
         <v/>
       </c>
       <c r="I25" s="52">
-        <f>IFERROR(MAX(0,MIN(167.63,I24+H25)),"")</f>
+        <f>IF(H25="","",MAX(0,MIN(167.63,I24+H25)))</f>
         <v/>
       </c>
       <c r="J25" s="56">
-        <f>IFERROR(MAX(0,H25-MAX(0,167.63-167.63)),"")</f>
+        <f>IF(H25="","",MAX(0,H25-MAX(0,167.63-I24)))</f>
         <v/>
       </c>
       <c r="K25" s="57" t="n"/>
@@ -2724,22 +2672,22 @@
       <c r="D26" s="59" t="n"/>
       <c r="E26" s="59" t="n"/>
       <c r="F26" s="60">
-        <f>IFERROR(SUM(B26:E26),"")</f>
+        <f>IF(COUNTA(B26:E26)=0,"",SUM(B26:E26))</f>
         <v/>
       </c>
       <c r="G26" s="61" t="n">
         <v>630</v>
       </c>
       <c r="H26" s="62">
-        <f>IFERROR(G26-F26,"")</f>
+        <f>IF(F26="","",G26-F26)</f>
         <v/>
       </c>
       <c r="I26" s="59">
-        <f>IFERROR(MAX(0,MIN(167.63,I25+H26)),"")</f>
+        <f>IF(H26="","",MAX(0,MIN(167.63,I25+H26)))</f>
         <v/>
       </c>
       <c r="J26" s="63">
-        <f>IFERROR(MAX(0,H26-MAX(0,167.63-167.63)),"")</f>
+        <f>IF(H26="","",MAX(0,H26-MAX(0,167.63-I25)))</f>
         <v/>
       </c>
       <c r="K26" s="2" t="n"/>
@@ -2755,22 +2703,22 @@
       <c r="D27" s="52" t="n"/>
       <c r="E27" s="52" t="n"/>
       <c r="F27" s="53">
-        <f>IFERROR(SUM(B27:E27),"")</f>
+        <f>IF(COUNTA(B27:E27)=0,"",SUM(B27:E27))</f>
         <v/>
       </c>
       <c r="G27" s="54" t="n">
         <v>630</v>
       </c>
       <c r="H27" s="55">
-        <f>IFERROR(G27-F27,"")</f>
+        <f>IF(F27="","",G27-F27)</f>
         <v/>
       </c>
       <c r="I27" s="52">
-        <f>IFERROR(MAX(0,MIN(167.63,I26+H27)),"")</f>
+        <f>IF(H27="","",MAX(0,MIN(167.63,I26+H27)))</f>
         <v/>
       </c>
       <c r="J27" s="56">
-        <f>IFERROR(MAX(0,H27-MAX(0,167.63-167.63)),"")</f>
+        <f>IF(H27="","",MAX(0,H27-MAX(0,167.63-I26)))</f>
         <v/>
       </c>
       <c r="K27" s="57" t="n"/>
@@ -2786,22 +2734,22 @@
       <c r="D28" s="59" t="n"/>
       <c r="E28" s="59" t="n"/>
       <c r="F28" s="60">
-        <f>IFERROR(SUM(B28:E28),"")</f>
+        <f>IF(COUNTA(B28:E28)=0,"",SUM(B28:E28))</f>
         <v/>
       </c>
       <c r="G28" s="61" t="n">
         <v>630</v>
       </c>
       <c r="H28" s="62">
-        <f>IFERROR(G28-F28,"")</f>
+        <f>IF(F28="","",G28-F28)</f>
         <v/>
       </c>
       <c r="I28" s="59">
-        <f>IFERROR(MAX(0,MIN(167.63,I27+H28)),"")</f>
+        <f>IF(H28="","",MAX(0,MIN(167.63,I27+H28)))</f>
         <v/>
       </c>
       <c r="J28" s="63">
-        <f>IFERROR(MAX(0,H28-MAX(0,167.63-167.63)),"")</f>
+        <f>IF(H28="","",MAX(0,H28-MAX(0,167.63-I27)))</f>
         <v/>
       </c>
       <c r="K28" s="2" t="n"/>
@@ -2817,22 +2765,22 @@
       <c r="D29" s="52" t="n"/>
       <c r="E29" s="52" t="n"/>
       <c r="F29" s="53">
-        <f>IFERROR(SUM(B29:E29),"")</f>
+        <f>IF(COUNTA(B29:E29)=0,"",SUM(B29:E29))</f>
         <v/>
       </c>
       <c r="G29" s="54" t="n">
         <v>630</v>
       </c>
       <c r="H29" s="55">
-        <f>IFERROR(G29-F29,"")</f>
+        <f>IF(F29="","",G29-F29)</f>
         <v/>
       </c>
       <c r="I29" s="52">
-        <f>IFERROR(MAX(0,MIN(167.63,I28+H29)),"")</f>
+        <f>IF(H29="","",MAX(0,MIN(167.63,I28+H29)))</f>
         <v/>
       </c>
       <c r="J29" s="56">
-        <f>IFERROR(MAX(0,H29-MAX(0,167.63-167.63)),"")</f>
+        <f>IF(H29="","",MAX(0,H29-MAX(0,167.63-I28)))</f>
         <v/>
       </c>
       <c r="K29" s="57" t="n"/>
@@ -2848,22 +2796,22 @@
       <c r="D30" s="59" t="n"/>
       <c r="E30" s="59" t="n"/>
       <c r="F30" s="60">
-        <f>IFERROR(SUM(B30:E30),"")</f>
+        <f>IF(COUNTA(B30:E30)=0,"",SUM(B30:E30))</f>
         <v/>
       </c>
       <c r="G30" s="61" t="n">
         <v>630</v>
       </c>
       <c r="H30" s="62">
-        <f>IFERROR(G30-F30,"")</f>
+        <f>IF(F30="","",G30-F30)</f>
         <v/>
       </c>
       <c r="I30" s="59">
-        <f>IFERROR(MAX(0,MIN(167.63,I29+H30)),"")</f>
+        <f>IF(H30="","",MAX(0,MIN(167.63,I29+H30)))</f>
         <v/>
       </c>
       <c r="J30" s="63">
-        <f>IFERROR(MAX(0,H30-MAX(0,167.63-167.63)),"")</f>
+        <f>IF(H30="","",MAX(0,H30-MAX(0,167.63-I29)))</f>
         <v/>
       </c>
       <c r="K30" s="2" t="n"/>
@@ -2879,22 +2827,22 @@
       <c r="D31" s="52" t="n"/>
       <c r="E31" s="52" t="n"/>
       <c r="F31" s="53">
-        <f>IFERROR(SUM(B31:E31),"")</f>
+        <f>IF(COUNTA(B31:E31)=0,"",SUM(B31:E31))</f>
         <v/>
       </c>
       <c r="G31" s="54" t="n">
         <v>630</v>
       </c>
       <c r="H31" s="55">
-        <f>IFERROR(G31-F31,"")</f>
+        <f>IF(F31="","",G31-F31)</f>
         <v/>
       </c>
       <c r="I31" s="52">
-        <f>IFERROR(MAX(0,MIN(167.63,I30+H31)),"")</f>
+        <f>IF(H31="","",MAX(0,MIN(167.63,I30+H31)))</f>
         <v/>
       </c>
       <c r="J31" s="56">
-        <f>IFERROR(MAX(0,H31-MAX(0,167.63-167.63)),"")</f>
+        <f>IF(H31="","",MAX(0,H31-MAX(0,167.63-I30)))</f>
         <v/>
       </c>
       <c r="K31" s="57" t="n"/>
@@ -2910,22 +2858,22 @@
       <c r="D32" s="59" t="n"/>
       <c r="E32" s="59" t="n"/>
       <c r="F32" s="60">
-        <f>IFERROR(SUM(B32:E32),"")</f>
+        <f>IF(COUNTA(B32:E32)=0,"",SUM(B32:E32))</f>
         <v/>
       </c>
       <c r="G32" s="61" t="n">
         <v>630</v>
       </c>
       <c r="H32" s="62">
-        <f>IFERROR(G32-F32,"")</f>
+        <f>IF(F32="","",G32-F32)</f>
         <v/>
       </c>
       <c r="I32" s="59">
-        <f>IFERROR(MAX(0,MIN(167.63,I31+H32)),"")</f>
+        <f>IF(H32="","",MAX(0,MIN(167.63,I31+H32)))</f>
         <v/>
       </c>
       <c r="J32" s="63">
-        <f>IFERROR(MAX(0,H32-MAX(0,167.63-167.63)),"")</f>
+        <f>IF(H32="","",MAX(0,H32-MAX(0,167.63-I31)))</f>
         <v/>
       </c>
       <c r="K32" s="2" t="n"/>
@@ -2941,22 +2889,22 @@
       <c r="D33" s="52" t="n"/>
       <c r="E33" s="52" t="n"/>
       <c r="F33" s="53">
-        <f>IFERROR(SUM(B33:E33),"")</f>
+        <f>IF(COUNTA(B33:E33)=0,"",SUM(B33:E33))</f>
         <v/>
       </c>
       <c r="G33" s="54" t="n">
         <v>630</v>
       </c>
       <c r="H33" s="55">
-        <f>IFERROR(G33-F33,"")</f>
+        <f>IF(F33="","",G33-F33)</f>
         <v/>
       </c>
       <c r="I33" s="52">
-        <f>IFERROR(MAX(0,MIN(167.63,I32+H33)),"")</f>
+        <f>IF(H33="","",MAX(0,MIN(167.63,I32+H33)))</f>
         <v/>
       </c>
       <c r="J33" s="56">
-        <f>IFERROR(MAX(0,H33-MAX(0,167.63-167.63)),"")</f>
+        <f>IF(H33="","",MAX(0,H33-MAX(0,167.63-I32)))</f>
         <v/>
       </c>
       <c r="K33" s="57" t="n"/>
@@ -2972,22 +2920,22 @@
       <c r="D34" s="59" t="n"/>
       <c r="E34" s="59" t="n"/>
       <c r="F34" s="60">
-        <f>IFERROR(SUM(B34:E34),"")</f>
+        <f>IF(COUNTA(B34:E34)=0,"",SUM(B34:E34))</f>
         <v/>
       </c>
       <c r="G34" s="61" t="n">
         <v>630</v>
       </c>
       <c r="H34" s="62">
-        <f>IFERROR(G34-F34,"")</f>
+        <f>IF(F34="","",G34-F34)</f>
         <v/>
       </c>
       <c r="I34" s="59">
-        <f>IFERROR(MAX(0,MIN(167.63,I33+H34)),"")</f>
+        <f>IF(H34="","",MAX(0,MIN(167.63,I33+H34)))</f>
         <v/>
       </c>
       <c r="J34" s="63">
-        <f>IFERROR(MAX(0,H34-MAX(0,167.63-167.63)),"")</f>
+        <f>IF(H34="","",MAX(0,H34-MAX(0,167.63-I33)))</f>
         <v/>
       </c>
       <c r="K34" s="2" t="n"/>
@@ -3003,22 +2951,22 @@
       <c r="D35" s="52" t="n"/>
       <c r="E35" s="52" t="n"/>
       <c r="F35" s="53">
-        <f>IFERROR(SUM(B35:E35),"")</f>
+        <f>IF(COUNTA(B35:E35)=0,"",SUM(B35:E35))</f>
         <v/>
       </c>
       <c r="G35" s="54" t="n">
         <v>630</v>
       </c>
       <c r="H35" s="55">
-        <f>IFERROR(G35-F35,"")</f>
+        <f>IF(F35="","",G35-F35)</f>
         <v/>
       </c>
       <c r="I35" s="52">
-        <f>IFERROR(MAX(0,MIN(167.63,I34+H35)),"")</f>
+        <f>IF(H35="","",MAX(0,MIN(167.63,I34+H35)))</f>
         <v/>
       </c>
       <c r="J35" s="56">
-        <f>IFERROR(MAX(0,H35-MAX(0,167.63-167.63)),"")</f>
+        <f>IF(H35="","",MAX(0,H35-MAX(0,167.63-I34)))</f>
         <v/>
       </c>
       <c r="K35" s="57" t="n"/>
@@ -3029,37 +2977,29 @@
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B37" s="65">
-        <f>SUM(B5:B17)</f>
-        <v/>
-      </c>
-      <c r="C37" s="65">
-        <f>SUM(C5:C17)</f>
-        <v/>
-      </c>
-      <c r="D37" s="65">
-        <f>SUM(D5:D17)</f>
-        <v/>
-      </c>
-      <c r="E37" s="65">
-        <f>SUM(E5:E17)</f>
-        <v/>
-      </c>
-      <c r="F37" s="65">
-        <f>SUM(F5:F17)</f>
-        <v/>
-      </c>
-      <c r="G37" s="65">
-        <f>630*13</f>
-        <v/>
-      </c>
-      <c r="H37" s="65">
-        <f>SUM(H5:H17)</f>
-        <v/>
-      </c>
-      <c r="J37" s="65">
-        <f>SUM(J5:J17)</f>
-        <v/>
+      <c r="B37" s="65" t="n">
+        <v>589.39</v>
+      </c>
+      <c r="C37" s="65" t="n">
+        <v>4130.96</v>
+      </c>
+      <c r="D37" s="65" t="n">
+        <v>505.8</v>
+      </c>
+      <c r="E37" s="65" t="n">
+        <v>241.67</v>
+      </c>
+      <c r="F37" s="65" t="n">
+        <v>5467.82</v>
+      </c>
+      <c r="G37" s="65" t="n">
+        <v>7560</v>
+      </c>
+      <c r="H37" s="65" t="n">
+        <v>2092.18</v>
+      </c>
+      <c r="J37" s="65" t="n">
+        <v>2092.18</v>
       </c>
     </row>
     <row r="38" ht="20" customHeight="1">
@@ -3068,36 +3008,35 @@
           <t>AVERAGES</t>
         </is>
       </c>
-      <c r="B38" s="59">
-        <f>IFERROR(B37/COUNTA(B5:B17),"")</f>
-        <v/>
-      </c>
-      <c r="C38" s="59">
-        <f>IFERROR(C37/COUNTA(C5:C17),"")</f>
-        <v/>
-      </c>
-      <c r="D38" s="59">
-        <f>IFERROR(D37/COUNTA(D5:D17),"")</f>
-        <v/>
-      </c>
-      <c r="E38" s="59">
-        <f>IFERROR(E37/COUNTA(E5:E17),"")</f>
-        <v/>
-      </c>
-      <c r="F38" s="59">
-        <f>IFERROR(F37/COUNTA(F5:F17),"")</f>
-        <v/>
-      </c>
-      <c r="H38" s="59">
-        <f>IFERROR(H37/COUNTA(H5:H17),"")</f>
-        <v/>
+      <c r="B38" s="59" t="n">
+        <v>49.12</v>
+      </c>
+      <c r="C38" s="59" t="n">
+        <v>344.25</v>
+      </c>
+      <c r="D38" s="59" t="n">
+        <v>42.15</v>
+      </c>
+      <c r="E38" s="59" t="n">
+        <v>20.14</v>
+      </c>
+      <c r="F38" s="59" t="n">
+        <v>455.65</v>
+      </c>
+      <c r="G38" s="59" t="n">
+        <v>630</v>
+      </c>
+      <c r="H38" s="59" t="n">
+        <v>174.35</v>
+      </c>
+      <c r="J38" s="59" t="n">
+        <v>174.35</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="2">
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A37"/>
   </mergeCells>
   <conditionalFormatting sqref="H5:H17">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">

</xml_diff>